<commit_message>
fix(watch-links): Excel turbo prints its summary, projects and changes one page wide
Fable's PDF check found Özet split across three pages. Özet, Projeler and Değişenler now print
landscape and one page wide; the 26-column link sheets print landscape unsqueezed, since one page
wide their text is unreadable on paper. Content unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PYXngKVhjE7rF32UcXMcjY
</commit_message>
<xml_diff>
--- a/.planning/research/watch-links/2026-10-08-whatsapp/turbo/Excel-turbo.xlsx
+++ b/.planning/research/watch-links/2026-10-08-whatsapp/turbo/Excel-turbo.xlsx
@@ -480,7 +480,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -779,6 +779,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -786,7 +787,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -1604,6 +1605,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
 
@@ -8607,6 +8609,7 @@
   </sheetData>
   <autoFilter ref="A1:Z64"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
 
@@ -21926,6 +21929,7 @@
   </sheetData>
   <autoFilter ref="A1:Z126"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
 </worksheet>
 </file>
 
@@ -21933,7 +21937,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:M81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
@@ -25939,5 +25943,6 @@
   </sheetData>
   <autoFilter ref="A1:M81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs(two-videos review): his two videos and one X post reviewed by two blind readers, merged at max; a new Excel sheet "Yeni eklenenler"
His order: the repos and skills of HhZdNYI4pJs, LCwT00LrPZg and RahulTechX's post,
reviewed the way the 88 links were, his five exclusions left out, no frame-by-frame.
Opus 5.5 high and Fable 5.1 high read blind; the lead switched itself to max through
operator and refereed eight splits (MERGE.md §2 — the method-class tools stay out on
his 2026-08-27 order; Claude Security's licence is Anthropic's own, not Apache-2.0).
Sonnet wrote the sheet: 34 rows, the five old sheets value-identical, desktop and repo
copies byte-identical. Nothing installed; each install waits on his word at its rank.
STATE's three headings rewritten.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FoxtQqqZvF98c8hzhQtwNW
</commit_message>
<xml_diff>
--- a/.planning/research/watch-links/2026-10-08-whatsapp/turbo/Excel-turbo.xlsx
+++ b/.planning/research/watch-links/2026-10-08-whatsapp/turbo/Excel-turbo.xlsx
@@ -12,11 +12,13 @@
     <sheet name="Öncelikli" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Tüm linkler" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Değişenler" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Yeni eklenenler" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Öncelikli'!$A$1:$Z$64</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Tüm linkler'!$A$1:$Z$89</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Değişenler'!$A$1:$M$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Yeni eklenenler'!$A$1:$N$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +45,17 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000563C1"/>
+      <sz val="11"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="7">
@@ -90,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -116,6 +129,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -21812,4 +21831,2375 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="58" customWidth="1" min="5" max="5"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="45" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="62" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Ad</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Bağlantı</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Hangi video</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Ne bu</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Gerçek mi (yıldız, son güncelleme, lisans)</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Elimizde var mı</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Holdingte yeri (sıra)</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>İnşaat ekibine</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Getirisi</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Onay gerekir</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Öneri (hakem)</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>Neden</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>YE01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Supabase Agent Skills (yalnız beceriler, MCP değil)</t>
+        </is>
+      </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/supabase/agent-skills</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>V1 07:01</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Supabase'in resmî iki becerisi. supabase: Auth, RLS, Edge Functions, migration ve güvenlik denetimi. supabase-postgres-best-practices: sorgu, index, bağlantı havuzu, kilitlenme ve RLS kuralları, etkiye göre sıralı.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Evet. 2.827 yıldız, son push 2026-10-02, MIT, resmî Supabase org. Dikkat: Anthropic pazarındaki supabase eklentisi başka bir şey (supabase-community'nin MCP'si, veritabanına dokunur). Alınacak olan yalnız becerilerdir, MCP değil.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Yok. Çalışma kartlarımız Supabase'in kendisi hakkında; beceriler hakkında kart yok.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>#3, #4 (tahtadan sonra sıradaki iş)</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Evet — yazan koltuklar (lider, helper-writer, builder)</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Makine. Holdingin bütün durumu tek bir Supabase/Postgres'te duruyor (STACK.md) ve ilk sekiz sıranın yarısı bu veritabanının güvenliği. Becerinin kuralları da tam olarak bu açıkları anlatıyor.</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Düşük; markdown bilgisi. MCP'si kurulmamalı: şirket veritabanı yalnız SELECT ile okunur.</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Kurulum</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>İki okuyucunun da ilk ikisinden biri. Yalnız beceriler alınır, MCP değil. Sıra 3 başlarken gerekir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>YE02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>The prompting playbook (Anthropic konuşması, X1)</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=G2B0YWuJUgI</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>X1 00:00–33:24 (RahulTechX gönderisi: https://x.com/RahulTechX/status/2110166431610572865; konuşmacı Margot Van Laar, Anthropic uygulamalı yapay zekâ mühendisi, Code with Claude Londra)</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Bir depo değil, bir konuşma. Anlattıkları şunlar: (1) önce değerlendirme seti: kontrol, kenar ve devretme vakaları; (2) XML ile düzen ve çıktı sözleşmesi, gerekirse modelin çevresindeki kodda durdurma dizisi; (3) eski modeller için eklenmiş savunma yamaları yeni modelde aşırı uygulanıp bilgi saklatıyor; her yama sebebiyle sürüm kontrolünde tutulmalı; (4) 'talimat yetenek eklemez': hesap için emir değil araç ver; (5) bir kuralın maliyetini yazıyorsan faydasını da yaz; (6) tek büyük prompt yerine üretim, değerlendirme ve onarım için üç ayrı prompt. Konuşmadaki örnekte bu yol, Opus'un uyarlanabilir düşünmesine göre daha az token ve daha düşük gecikmeyle bütün testleri geçti.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Konuşma gerçek ve Anthropic'in; Claude kanalında 2026-05-22'den beri herkese açık (152.901 izlenme). Gönderinin hikâyesi yanlış: 'hiç çıkmaması gereken video' değil. Gönderideki makale (x.com/i/article/2073973224455733248): Opus bunu yalnız genel bir 'LLM nasıl eğitilir' yazısı buldu, Fable açamadı (404); iki durumda da içinde araç yok.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Fikirlerin bir kısmı zaten bizde: kör A/B testi, W101 'kontroller geçmeden kart kapanmaz', dxb-verify. Persona ve Hamza prompt'larının eski model yamaları açısından taranması ise hiçbir satırda yok (aranmadı; olmadığı iddia edilmiyor, yalnız ORDER ve MERGE'de görülmedi).</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>#11, #13, #16</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Persona ve Hamza-bağlam koltukları (bilgi olarak; kurulacak bir şey yok)</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Makine. Opus 5'ten 5.5'e geçişte prompt'larda kalan yamaları bulmak için bir yöntem.</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Bir kapı satırı yalnız sizin sözünüzle</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Bilgi; kurulacak bir şey yok. X1'deki 'sızdırılmış' video Anthropic'in herkese açık konuşmasıdır (The prompting playbook, Claude kanalı, G2B0YWuJUgI, 2026-05-22).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>YE03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>HyperFrames (HeyGen)</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/heygen-com/hyperframes</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>V1 00:26 · V2 11:20</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>HTML, CSS ve animasyondan birebir aynı MP4'ü üreten açık kaynak bir çerçeve. Headless Chrome kareyi çizer, FFmpeg kodlar. Claude Code eklentisi ve beceri seti de var.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Evet. 63.591 yıldız, son push 2026-10-14, Apache-2.0. Anthropic'in resmî eklenti pazarında da hyperframes adıyla duruyor (yerel kopyada ölçüldü). Gereken Node 22+ (bizde v22.23.2), FFmpeg (~/.local/bin/ffmpeg) ve Chrome (/usr/bin/google-chrome); üçü de makinede var. 'Render başına ücret yok' sözü doğru: yerel çekirdek ücretsiz, HeyGen'in bulut ve avatar tarafı ayrıca ücretli. V2'deki 'bu videonun bütün hareketli grafikleri HyperFrames ile yapıldı' sözü yaratıcının iddiası; doğrulanmadı.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Yok, kurulu değil. Çalışma kartı var (study-cards/heygen-hyperframes.md, STUDY, meşruiyet OK). Zaten MERGE ve ORDER'da: W025 ve sıra #45 (B43).</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>#45 (B43 stüdyo) → #46, #49</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Hayır (stüdyo)</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>İkisi de. Ekran kartını kullanmadığı için B33'ün kart kuyruğuna girmez. Kanal tanıtımları, başlık kartları, altyazı ve açıklayıcı videoları GPU'suz üretir. MERGE'deki 16 numaralı gelir fikri, helal-finans açıklayıcıları, doğrudan buna dayanır.</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Hazır şablonlarda müzik ya da görsel olabilir; Y4 helal ekranından (#5) geçmeli. Sürüm hızlı değişiyor, bu yüzden sürüm sabitlenmeli.</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Kurulum</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Al</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>Stüdyonun eli, inşaat oturumunun aleti değil; tezgâhta #45'te kurulur.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>YE04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Claude Security (Anthropic eklentisi)</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/anthropics/claude-plugins-official/tree/main/plugins/claude-security</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>V1 08:12</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Oturumun içinde bir ajan ekibi çalıştırır: mimariyi çıkarır, tehdit modeli kurar, açık arar ve her bulguyu ayrı bir ajanla doğrular. İstenirse yama dosyası önerir. Anthropic'in barındırılan 'Claude Security' ürününün oturum içi sürümüdür.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Evet. Resmî eklenti pazarı deposu 38.048 yıldız (Apache-2.0); eklenti klasörü 2026-09-25'te güncellendi. Eklentinin lisansı: Anthropic, tüm hakları saklı (pazar deposu Apache-2.0, eklentinin kendisi değil). Yerel pazar kopyasında mevcut (~/.claude/plugins/marketplaces/claude-plugins-official/plugins/claude-security). README Opus 5.5 veya Fable 5.1 öneriyor; taramanın bazı kısımları Opus 4.8'e düşebiliyor. Kendi yalıtımı yok.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Kurulu değil. Yerleşik /security-review becerisi daha hafif bir ikiz.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>#4; sonra #32 ve #51</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Evet — liderin koltuğu, her seferinde tek tarama</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Makine. Bulguları ikinci bir ajan doğruluyor; bu, bizim 'ölçmeden söyleme' kuralımızla aynı yapı.</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Token maliyeti (tarama önce maliyeti sorup onay alıyor). Doktrin 1-bis gereği, açılmadan önce kancaları ölçülmeli.</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Kurulum; taramanın efor kademesi</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Dene</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Bir iş yapıyor, yöntem sınıfı değil (1-ter ona dokunmaz). Önce #4'te inşaat kopyasında tek tarama; kendini kanıtlarsa #32 ve #51. Eklenti Claude Code içinde kullanılır, holdinge kopyalanmaz. 3 kancası var (hooks.json: açılış yazısı, kendi betiklerinden sonra kullanım sayımı, git push sonrası tarama ipucu); doktrin 1-bis gereği hooks.py açılmadan önce okunur — 14 Ekim 2026 gecesi okunmadı.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>YE05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Playwright CLI (Microsoft)</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/microsoft/playwright-cli</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>V1 07:52</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Playwright'ın komut satırı yüzü. Ajan, sayfayı kısa komutlarla açar, tıklar ve ekran görüntüsü alır. MCP'nin aksine sayfa ağacını modele dökmez.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Evet. 14.177 yıldız, son push 2026-10-14, Apache-2.0, resmî Microsoft. 'Token'da daha hafif' sözü README'nin kendi iddiası; bizde ölçülmedi.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>İkizlerimiz var. Playwright MCP bağlı (mcp__playwright__*), playwright eklentisi kurulu ama kapalı, B35'te Playwright headless eli var.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>#15 (B35), #16</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Evet — dxb-verify'ın tarayıcı kontrolleri</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Makine. Ekran doğrulaması daha ucuz olur; 2.4 milyon token dersinin konusu tam bu.</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Düşük. Elimizdeki MCP ile ikilik yaratır; ölçüm sonucu hangisinin kalacağını seçer.</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Kurulum</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Dene</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>Playwright MCP'ye karşı tek bir gerçek kontrolde ölçülür. 'Token'da daha hafif' sözü burada ölçülmedi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>YE06</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Google Workspace CLI (gws)</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/googleworkspace/cli</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>V1 01:28</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Drive, Gmail, Takvim, Sheets, Docs ve diğer Workspace API'leri için tek bir komut satırı aracı. Komutlarını Google'ın Discovery servisinden çalışırken kurar. İçinde 40'tan fazla ajan becerisi var (gws-gmail-send, gws-sheets-append …).</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Evet. 31.497 yıldız, son push 2026-10-06, Apache-2.0. Ama README açıkça resmî olarak desteklenen bir Google ürünü olmadığını söylüyor ve 1.0 öncesi olduğu için kırıcı değişiklik bekleniyor. Giriş için bir Google Cloud projesi ve OAuth gerekiyor.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Yok. Yakın bir ikizimiz var: outbox-executor'daki tek Gmail-gönderme yetkisi (packages/outbox-executor/src/actions/email-send-staging.ts).</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>#24 (+ #52 B05)</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>#24'e kadar hayır</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Makine tarafında, Resepsiyon'un gelen postayı okuyup dosyalaması için hazır bir el olur.</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Kimlik ve yetki adımı gerektirir; OAuth kapsamı geniş tutulursa hesabın tamamı açılır. Resmî Google ürünü değil ve henüz 1.0 öncesi.</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Kurulum + Google Cloud/OAuth (kimlik adımı)</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Dene</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>Resmî Google ürünü değil, 1.0 öncesi (README); OAuth ve Cloud projesi sizin kimlik adımınız. #24'ten önce kurulsa boşta durur — tezgâh kuralınız. #24'te denenir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>YE07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>CodeBurn</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/getagentseal/codeburn</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>V1 09:27</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Claude Code dahil 37 aracın diskteki oturum kayıtlarını okuyup token harcamasını modele, projeye ve göreve göre gösteren yerel bir araç. Her mesajda yüklenen ama hiç kullanılmayan MCP gibi israfı işaretler.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Evet. 11.446 yıldız, son push 2026-10-14, MIT. README'ye göre CLI dışarıya hiçbir şey göndermiyor; yalnız fiyat listesini günde bir kez LiteLLM'den çekiyor. codeburn quota saklı kimlik bilgileriyle sağlayıcıya soru soruyor; share --pair LAN'a açılıyor.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Kısmi ikizler var: dxb-ctx bağlam ölçeri (yalnız oturum içi) ve LiteLLM maliyet defteri (şirket tarafında). İnşaat oturumlarının harcamasını proje ve görev bazında gösteren bir aracımız yok.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>#37'nin (B34) yanında</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Evet — lider, bir kez</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Makine: inşaat maliyeti tahminle değil ölçümle konuşulur.</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>quota ve share komutları kullanılmamalı.</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>npx indirmesi</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>Dene</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>Tek, salt okur koşu: quota ve share hiç kullanılmaz. Rakamları burada ölçülmedi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>YE08</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Humanizer</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/blader/humanizer</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>V1 04:18</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Yapay zekâ ile yazılmış metindeki kalıpları ('X değil, Y', üçlü sıralamalar, abartı kelimeleri) temizleyen bir beceri. Wikipedia'nın yapay zekâ yazısı belirtileri rehberine dayanır.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Evet. 56.924 yıldız, son push 2026-09-28, MIT. README'nin kendisi dedektörlerin çıktısının çoğunu hâlâ işaretlediğini söylüyor; yani amaç dedektörü atlatmak değil, okunurluk. Kalıplar yalnız İngilizce için yazılmış.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Yok. Çalışma kartı var (study-cards/humanizer.md, STUDY, meşruiyet OK). İkizi: B43'ün içerik becerisi ve W035'in yazım kuralları (ORDER #45).</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>#45; sonra #24 ve #47</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Hayır (satış koltukları)</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Gelir. İngilizce kanal anlatımı, soğuk e-posta ve site metni 'yapay zekâ kokmaz'.</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Türkçe kapsamı yok. Ses tonunu düzleştirebilir; testin ölçeceği şey de bu.</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Kurulum</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Dene</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>Sizin kör testiniz (a47543aa) karar verir: Humanizer ile No AI Slop'tan biri kalır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>YE09</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>No AI Slop</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/petergyang/no-ai-slop</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>V2 06:28</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>20'den fazla yapay zekâ yazı kalıbını temizleyen bir beceri. Sesi düzleştirmemeyi hedefler ve neyi değiştirdiğini listeler.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Evet. 12.365 yıldız, son push 2026-09-02, MIT. Video '22 kalıp' diyor; README '20+' diyor.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Yok. İkizi Humanizer ve W035.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>#45; sonra #24 ve #47</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Hayır (satış koltukları)</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Gelir, Humanizer ile aynı yoldan.</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Yalnız İngilizce.</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Kurulum</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Dene</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>Sizin kör testiniz (a47543aa) karar verir: Humanizer ile No AI Slop'tan biri kalır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>YE10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Apify MCP Server</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/apify/apify-mcp-server</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>V1 02:16</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Ajanı Apify Store'daki binlerce hazır kazıyıcıya ('Actor') bağlayan bir MCP sunucusu. Sunucu açık kaynak, kazıyıcılar ise Apify'ın bulutunda çalışır.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Evet. 11.220 yıldız, son push 2026-10-14, MIT. Ücretsiz plan ayda 5 $ ön ödemeli platform kullanımı; bu rakam apify.com/pricing sayfasında ölçüldü.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>İkizlerimiz kurulu: Agent-Reach, Scrapling ve MediaCrawler (B30). Çalışma kartı var (study-cards/apify.md, STUDY). Zaten MERGE'de: W014 → Y9 müşteri bulma (#48) ve B30.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>#48</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Gelir. Instagram ve TikTok'ta ücretsiz araçların takıldığı yerde müşteri listesi çıkarır.</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Para çıkışı (sonuç başına ücret). Ham liste satışı ve KVKK yasağı MERGE'de yazılı.</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Hesap (kimlik adımı), para çıkışı</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>İzle</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>Sonuç başına para çıkışı; ücretsiz ikizler (Scrapling) önce. Yalnız Scrapling'in yetmediği yerde #48'de denenir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>YE11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Expo Skills</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/expo/skills</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>V1 06:23</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Expo ekibinin resmî becerileri: React Native uygulamasını kurmak, EAS ile yayınlamak, sürüm yükseltmek.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Evet. 2.850 yıldız, son push 2026-10-14, MIT, resmî. Anthropic pazarında expo adıyla duruyor.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Yok.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Tahtada yeri yok (fikir 22 → B17, #50)</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 itibarıyla yok.</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Apple geliştirici hesabı yıllık 99 $; bu para çıkışı ve kimlik adımıdır.</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Apple hesabı, yılda 99 $</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>İzle</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>Tahtada yeri yok; yalnız fikir 22 (B17, #50) açılırsa gündeme gelir. Apple hesabı yılda 99 $.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>YE12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Stripe Best Practices (stripe/ai içindeki beceri)</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/stripe/ai/tree/main/skills/stripe-best-practices</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>V1 07:19</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Stripe entegrasyon kararları için resmî beceri: Checkout ile PaymentIntents arasında seçim, sandbox, webhook doğrulama, anahtar yetkileri, vergi.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Evet. Repo 1.940 yıldız, son push 2026-10-14, MIT. Beceri klasörü 2026-10-10'da güncellendi. Videonun 'tam eklentiyi değil yalnız bu beceriyi kur' uyarısı makul: tam eklenti providers/claude/plugin.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Yok. Çalışma kartı var (study-cards/stripe-mcp.md, STUDY).</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>#52 (B05)</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>B05'e kadar hayır</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Gelir: para girişinin güvenli yolu (fiyatın tarayıcıdan gelmemesi, webhook imzası).</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Stripe'ın kredi, taksit ve Treasury gibi ürünleri faizle ilişkilidir; riba eleği gerekir.</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Stripe hesabı (kimlik adımı)</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>İzle</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>B05 (#52) açılana kadar bekler; Stripe hesabı bir kimlik adımıdır.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>YE13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>OpenSEO</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/every-app/open-seo</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>V1 08:38</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Semrush ve Ahrefs'e açık kaynak bir alternatif: anahtar kelime, sıralama, backlink ve site denetimi. MCP ve beceriler içerir. Veriyi kullanıcının kendi DataForSEO anahtarıyla çeker.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Evet. 23.603 yıldız, son push 2026-10-14, MIT. Videonun 'veri onların sunucusunda kalır' sözü barındırılan sürüm için doğru; kendin barındırırsan (Docker veya Cloudflare) veri sende kalır. Barındırılan sürüm, DataForSEO isteklerinin üstüne %28 ekliyor (README).</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Yok. Zaten ORDER'da: #14 (B41'in satış dilimi) ve #40. MERGE X-21: kendi siteden sonra DataForSEO 50 $.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>#14/#47</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Gelir. Yerel SEO ve AEO hizmeti (MERGE fikir 7-8).</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>DataForSEO para çıkışıdır.</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Zaten tahtada</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>Zaten sırada: #14/#47. Yeni tahta satırı gerekmez; tahta yazılırken ilgili sıra bunu üstlenir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>YE14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Open Design</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/nexu-io/open-design</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>V2 15:46</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Claude Design'a açık kaynak, yerelde çalışan bir alternatif. Prototip, ekran ve sunum çizer; beceriyle genişletilebilir.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Evet. 101.156 yıldız, son push 2026-10-14, Apache-2.0.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Zaten var, open-design@open-design eklentisi kurulu ama kapalı (claude plugin list). Zaten MERGE'de: W025, W040 → B32.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>#21</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Makine: V2 taslakları.</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-19'da bağlanamadı (M-12); 2026-10-14'te yeniden ölçülmedi.</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Zaten var</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>Zaten kurulu (kapalı); yeri tahtada: #21. Yeni tahta satırı gerekmez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>YE15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>autoresearch (Karpathy)</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/karpathy/autoresearch</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>V2 16:07</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Bir ajanın tek bir GPU'da küçük bir dil modeli eğitim kodunu değiştirip 5 dakika eğitmesi, sonucun daha iyi olup olmadığına bakması ve iyiyse tutup kötüyse atması döngüsü. Talimatlar program.md'de.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Repo gerçek: 97.908 yıldız, son push 2026-03-26, lisans dosyası yok (GitHub lisans alanı boş). Ama videonun beceri diye anlattığı şey bir beceri değil, bir model eğitimi düzeneği. Videodaki spor programı örneği yalnız yöntemi bir prompt'la uyguluyor.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Çalışma kartı var: kurulu değil ve kurulmayacak. Zaten ORDER'da: #28 C40 (sabit bir skora karşı 'iyiyse tut' döngüsü, kalite kapısının dışında).</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>#28</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Makine: yöntem #28'de zaten yazılı.</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Zaten tahtada</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>Zaten sırada: #28. Yeni tahta satırı gerekmez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>YE16</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>ScrollCraft</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/nateherkai/scroll-craft</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>V1 03:08 (videoyu yapanın kendi aracı; videoda bunu açıkça söylüyor)</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Kaydırmayla ilerleyen, sinematik web sayfaları kuran bir ajan becerisi. Bir kaydırma motoru, tasarım kuralları ve kaydırmayı ekran görüntüsüyle denetleyen bir kontrolcü içerir.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Evet. 3.419 yıldız, son push 2026-09-30, MIT. Açıklamadaki 'ücretsiz' bağlantı bir e-posta toplama sayfasına gidiyor, ama GitHub deposu herkese açık.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Zaten var. ~/.claude/skills/scrollcraft kurulu; changelog'un son girdisi 2026-08-23. Üst kaynak bizdeki sürümden yeni.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>#42/#47</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Gelir. MERGE'deki 13 numaralı fikir: premium kaydırma siteleri.</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Yok, yalnız sürüm kayması.</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Zaten var</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>Zaten kurulu; üst kaynak farkı #42'de (W078), kendi sitemiz #47'de. Yeni tahta satırı gerekmez.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>YE17</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>claude-mem (videoda 'şimdilik bekleyin' uyarısıyla geçiyor)</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/thedotmack/claude-mem</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>V1 09:36</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Oturumlar arası hafıza eklentisi.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Videonun 'kullanım verisi gönderiyor' sözü doğru. Kendi dokümanı (docs/public/telemetry.mdx): varsayılan olarak açık, kapatmak kullanıcıya bırakılmış; PostHog'a anonim kurulum kimliği, model adı ve fatura katmanı gidiyor. Bu makinede ölçüldü: ~/.claude-mem/telemetry.json içinde decidedAt boş (karar verilmemiş), DO_NOT_TRACK tanımsız, sürüm 13.16.0 açık. Dokümana göre bu durumda telemetri açık; gönderim trafiği ayrıca ölçülmedi. Depo (Fable'ın ölçümü): 100.729 yıldız, son push 2026-10-13, Apache-2.0.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Zaten var ve açık.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Makinenin kullanım bilgisi dışarı gidiyor (anonim).</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Tek satır: telemetrisi kapatılsın mı?</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Zaten var</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>Zaten kurulu. Telemetri bu makinede varsayılan olarak açık (13.16.0; decidedAt boş, DO_NOT_TRACK ve CLAUDE_MEM_TELEMETRY tanımsız); iki okuyucu da açık ölçtü. Öneri: kapatın (CLAUDE_MEM_TELEMETRY=0). PostHog olaylarının neyi taşıdığı kodda okunmadı.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>YE18</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Matt Pocock skills</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/mattpocock/skills</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>V1 06:12 · V2 10:05 (V2'nin 'işletim sistemi' dediği, 4. sıra)</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Küçük, bileşik beceriler; skills/engineering altında 19 tane: code-review, tdd, to-spec, implement, diagnosing-bugs, domain-modeling, codebase-design, wayfinder, retro… Yazarın sözü: süreci ele geçiren GSD/BMAD/Spec-Kit'in tersine denetim sende kalır.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>291.045 yıldız, son push 2026-10-13, MIT, 177 sorun kaydı. V2'nin kullanım biçimi (Fable orkestra, Sonnet yazar, dönmeden önce code-review ile kendi işini denetler) tam dxb-team2'nin lider/yardımcı/Sol şekli.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Yok; yerleşik code-review becerisi, Sol geçişi ve rakip-istihbarat 02'de '17 geliştirme iş akışı becerisi' satırı var.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Yeri yok</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Makine: yardımcının kendi çıktısını lidere dönmeden denetlemesi — Sol'a giden hata sayısı düşer (ölçülecek).</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Üçüncü taraf beceri ajan davranışını değiştirir — dosyalar kurulmadan okunur (SkillSpector kapısı).</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Yeniden açmak yalnız sizin sözünüzle</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>1-ter emriniz (CAPABILITY_ARSENAL_DOCTRINE.md satır 167-181, 2026-08-27), ürünü bir çalışma yöntemi olan eklentiyi dışarıda bırakır; yazar bunu GSD/BMAD/Spec-Kit'in alternatifi diye sunuyor, yani kendi sözüyle aynı sınıf. Yeniden açmak yalnız sizin sözünüzle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>YE19</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Agent Skills (Addy Osmani)</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/addyosmani/agent-skills</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>V1 05:23</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>25 mühendislik becerisi: /spec → /plan → /build → /test → /review → /ship zinciri; spec'i dosyaya yazar, oturum dağılınca yeni oturum kaldığı yerden sürer; spec adımı kenar durumlarını (çifte rezervasyon, iade, saat dilimi) sorar.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>106.633 yıldız, son push 2026-10-13, MIT, 118 sorun kaydı. Yazarın 'Anthropic'te Claude Code'da çalışıyor' sözü ölçülmedi (GitHub profiline bakılmadı).</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>İkizi var: .planning (GSD durumu), dxb-team2 (plan → yaz → doğrula → Sol), dxb-verify. Tracker'da vercel skills / agent-skills kartı ayrı bir şey (Vercel'inki).</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Yeri yok</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Makine: holdingin kendi mühendis ajanları (B64 adım 2'den sonra iş yaparken) için hazır süreç.</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Oturumda iki süreç aynı anda; 'spec' dosyaları planın tek kopyası kuralıyla çakışır.</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Yeniden açmak yalnız sizin sözünüzle</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>/spec → /ship bir çalışma yöntemidir (1-ter).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>YE20</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>pstack (Lauren Tan, @poteto)</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/cursor/plugins/tree/main/pstack</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>V2 02:12 (8. sıra)</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Cursor'da React compiler ekibinden Lauren Tan'ın her gün kullandığı beceri yığını; poteto-mode hedefe göre iş akışını seçer; ilke: 'önce bir ajanı titiz yap, sonra paralel koş'; çok modelli inceleme panelleri. Claude Code portu: https://github.com/michael-denyer/pstack-claude</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Asıl depo cursor/plugins 11.368 yıldız (pstack klasörü MIT, Lauren Tan); port pstack-claude 1.995 yıldız, MIT, son push 2026-10-14; open-pstack 415 yıldız. Video 'Pistak/potato' diye söylüyor, ad pstack.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>İkizi var: dxb-team2 (lider her parçayı doğrular), Kanun D (önce taslak), Sol geçişi (ikinci model paneli).</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Yeri yok</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Fikir olarak: paralel yazar açmadan önce tek yazarın güvenilirliğini ölçmek — kapıda var.</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Yeniden açmak yalnız sizin sözünüzle</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>Aynı kural (yöntem sınıfı, 1-ter); pstack ayrıca bir Cursor eklentisi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>YE21</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>unlazy</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/Leonxlnx/unlazy</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>V2 14:45 (listeye girmeyen dört beceriden ilki)</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Kabul defteri önce yazılır, koşturulabilir kapılar, dönen iş yeniden doğrulanır, yalnız kanıtın desteklediği rapor edilir; Depth Tree yöntemi (her yaprağa tam zaman bütçesi). Sürüm 2.1.0, etiketli yayın yok ('commit sabitleyin').</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>3.931 yıldız, son push 2026-09-03, MIT, 10 sorun kaydı. Araştırma dayanağı README'de listelenmiş, okunmadı.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>İkizi var: dxb-verify (kanıt önce 'bitti'), W101 tamamlanma sözleşmesi (sıra 9 Y7, sıra 16).</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Yeri yok</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Yeniden açmak yalnız sizin sözünüzle</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>Aynı kural (yöntem sınıfı, 1-ter).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>YE22</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Superpowers</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/obra/superpowers</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>V1 06:05 · V2 09:51</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Bir çalışma yöntemi eklentisi (dxb-team2'nin ikizi); iki videoda da yalnız adı geçti, ayrıca incelenmedi.</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>299.115 yıldız, MIT. Son güncelleme tarihi okuyucu raporlarında yok.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Yok; makineden kaldırıldı. 2026-08-27 emrinizde adıyla geçiyor. İkizi dxb-team2.</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Yeri yok</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Yeniden açmak yalnız sizin sözünüzle</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>Yöntem sınıfı; 2026-08-27 tarihli emriniz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>YE23</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Vibe Security (vibe-security-skill)</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/raroque/vibe-security-skill</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>V2 03:30</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Vibe-code ile yazılmış uygulamalardaki tipik açıkları arayan bir beceri: koda gömülü anahtar, atlanmış RLS, fiyatın istemciden gelmesi, localStorage'da duran token. Kurallar teknolojiye göre ayrı dosyalarda.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Evet, ama bakımsız. 1.122 yıldız (video 'binin altında' diyor, artık üstünde), MIT, son push 2026-03-15 (yedi ay önce).</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>İkizleri: Claude Security, Supabase becerisi, /security-review.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Yeri yok</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Makine, az. Supabase ve Next.js maddeleri bizim yığınımıza uyuyor.</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>Eski kalmış olabilir.</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>Son push 2026-03-15; Claude Security ile Supabase becerileri bunu karşılıyor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>YE24</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>RTK (Rust Token Killer)</t>
+        </is>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/rtk-ai/rtk</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>V1 09:01 (olumsuz: JetBrains testinde kazanç yok, düşük eforda daha pahalı)</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Komut çıktılarını kısaltan Rust vekil CLI; '%60-90 token' iddiası.</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>83.366 yıldız, son push 2026-10-14, Apache-2.0. Videonun aktardığı JetBrains testi bizce ölçülmedi.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Yok. Bash'in önünde zaten kendi kapılarımız var (dxb-cost-gate, dxb-prompt-gate).</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Yeri yok</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>Yeri yok; iki okuyucu da 'alma' dedi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>YE25</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Context Mode (context-mode)</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/mksglu/context-mode</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>V1 09:43 (video: 'açık hata kotayı yakıyor')</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Araç çıktısını sanal kutuya alıp bağlamı küçülten MCP + kanca katmanı, oturum hafızası.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>28.993 yıldız, son push 2026-10-14, lisans NOASSERTION (standart dışı), 359 açık sorun kaydı.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Yok; claude-mem aynı yerde duruyor.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Yeri yok</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>Yeri yok; iki okuyucu da 'alma' dedi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>YE26</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Firecrawl</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/firecrawl/firecrawl</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>V1 03:01</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Sayfa kazıma aracı; videoda yalnız anıldı, ayrıca incelenmedi.</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>191.543 yıldız, AGPL-3.0. Son güncelleme tarihi okuyucu raporlarında yok.</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Yok; ikizleri Scrapling ve Agent-Reach kurulu. W049'da zaten işlenmiş.</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Yeri yok</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>Yeri yok; iki okuyucu da 'alma' dedi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>YE27</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Remotion</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/remotion-dev/remotion</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>V1 01:03 · V2 11:28</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Videoyu kodla üreten bir çerçeve; iki videoda da yalnız anıldı, ayrıca incelenmedi.</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>64.095 yıldız; lisans NOASSERTION (şirketler için ücretli lisans modeli). Son güncelleme tarihi okuyucu raporlarında yok.</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Yok. Daha önce reddedilmiş (şirket lisansı; W071 ve video düzenleme araç zinciri kararı).</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Yeri yok</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>Yeri yok; iki okuyucu da 'alma' dedi. HyperFrames seçilirse Remotion'a yer kalmıyor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>YE28</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>AI Job Search</t>
+        </is>
+      </c>
+      <c r="C29" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/MadsLorentzen/ai-job-search</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>V2 15:24</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Bir kişinin kendi iş başvurularını yürütmesi için Claude Code üstünde bir iskelet: ilanı değerlendirir, CV ve ön yazı hazırlar.</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Evet. 46.795 yıldız, son push 2026-10-08, MIT.</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Yok.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>Yeri yok (holding iş aramıyor)</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Yok.</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>Yeri yok; iki okuyucu da 'alma' dedi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>YE29</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>HubSpot 'Claude at Work' rehberi (sponsor içeriği)</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>https://clickhubspot.com/f02a35</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>V2 05:35 (sponsor bölümü)</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Claude ürünlerinin haritası ve üç iş akışı; araç değil, sponsor içeriği. STACK HubSpot CRM'i dışlıyor.</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Videonun sponsoru; bağlantı bir e-posta toplama sayfası. Depo yok (yıldız ve lisans yok).</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>Yeri yok</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>Yeri yok; videonun sponsor içeriği.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>YE30</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>taste (taste-skill)</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
+      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="2" t="n"/>
+      <c r="I31" s="2" t="n"/>
+      <c r="J31" s="2" t="n"/>
+      <c r="K31" s="2" t="n"/>
+      <c r="L31" s="2" t="n"/>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>Hariç (sizin sözünüzle)</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>YE31</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>impeccable</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n"/>
+      <c r="D32" s="2" t="n"/>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="n"/>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="n"/>
+      <c r="I32" s="2" t="n"/>
+      <c r="J32" s="2" t="n"/>
+      <c r="K32" s="2" t="n"/>
+      <c r="L32" s="2" t="n"/>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>Hariç (sizin sözünüzle)</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>YE32</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>caveman</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="n"/>
+      <c r="D33" s="2" t="n"/>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="n"/>
+      <c r="G33" s="2" t="n"/>
+      <c r="H33" s="2" t="n"/>
+      <c r="I33" s="2" t="n"/>
+      <c r="J33" s="2" t="n"/>
+      <c r="K33" s="2" t="n"/>
+      <c r="L33" s="2" t="n"/>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>Hariç (sizin sözünüzle)</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>YE33</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>ponytail</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="n"/>
+      <c r="D34" s="2" t="n"/>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="n"/>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="n"/>
+      <c r="I34" s="2" t="n"/>
+      <c r="J34" s="2" t="n"/>
+      <c r="K34" s="2" t="n"/>
+      <c r="L34" s="2" t="n"/>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>Hariç (sizin sözünüzle)</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>YE34</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Agent-Reach</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="n"/>
+      <c r="D35" s="2" t="n"/>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="n"/>
+      <c r="G35" s="2" t="n"/>
+      <c r="H35" s="2" t="n"/>
+      <c r="I35" s="2" t="n"/>
+      <c r="J35" s="2" t="n"/>
+      <c r="K35" s="2" t="n"/>
+      <c r="L35" s="2" t="n"/>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>Hariç (sizin sözünüzle)</t>
+        </is>
+      </c>
+      <c r="N35" s="2" t="n"/>
+    </row>
+    <row r="36"/>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>Kaynak: iki video (Nate Herk, Dubibubi) ve RahulTechX gönderisi; okuyucular Opus 5.5 ve Fable 5.1, hakem Opus 5.5 max, 14 Ekim 2026. Hiçbir şey sizin sözünüz olmadan kurulmaz.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N35"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId29"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(watch-links): WhatsApp links since 5 Oct — seven new ones reviewed into a new Excel sheet "Ekim 9-15 linkleri"
Already-reviewed items (W121-W125, apple-design, the two Voxyz posts of 13 Oct) skipped on his word.
Nothing installed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NB6Ab2cUJEAKN9Gac26UTy
</commit_message>
<xml_diff>
--- a/.planning/research/watch-links/2026-10-08-whatsapp/turbo/Excel-turbo.xlsx
+++ b/.planning/research/watch-links/2026-10-08-whatsapp/turbo/Excel-turbo.xlsx
@@ -13,6 +13,7 @@
     <sheet name="Tüm linkler" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Değişenler" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Yeni eklenenler" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Ekim 9-15 linkleri" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Öncelikli'!$A$1:$Z$64</definedName>
@@ -24158,7 +24159,6 @@
       </c>
       <c r="N35" s="2" t="n"/>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
         <is>
@@ -24202,4 +24202,682 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="58" customWidth="1" min="5" max="5"/>
+    <col width="62" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="45" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="62" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Ad</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Bağlantı</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Hangi video</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Ne bu</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Gerçek mi (yıldız, son güncelleme, lisans)</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Elimizde var mı</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Holdingte yeri (sıra)</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>İnşaat ekibine</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Getirisi</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Onay gerekir</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Öneri (hakem)</t>
+        </is>
+      </c>
+      <c r="N1" s="4" t="inlineStr">
+        <is>
+          <t>Neden</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>EK01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>callanxai — 'Karpathy: Prompting bitiyor, Graph kalıyor'</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/callanxai/status/2108285248223986139</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>69 dk video; döküm tamamı</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Karpathy'nin 2023'teki iki Stanford konuşması birbirine eklenmiş: bir hackathon açılışı ve 'Transformer'a giriş' dersi. Arada başka bir konuşmacıdan kısa bir parça var.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Başlık yalan, hatta tersini söylüyor. Karpathy prompt'u 'yeni programlama' diye övüyor (20:28, 20:48). 'Delete everything' sözü (39:48) 'delete everything, keep attention' cümlesinin parçası; RNN'leri atıp attention'ı tutmaktan bahsediyor. 'Graph' yalnız transformer'ın iç yapısı anlamında geçiyor.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Kaynak güvenilmez</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Eski bir ders, sahte başlıkla paylaşılmış.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>EK02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>hayatomaruu — 'Anthropic mühendisi: 100+ ajan döngüde'</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/hayatomaruu/status/2108329507442565186</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>27 dk webinar; döküm tamamı</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic çalışanının Claude Code'da token tasarrufu webinarı. Konuları: önbellek, /usage, /compact, CLAUDE.md ile becerilerin ayrılması, yönetici ayarları.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Konuşma gerçek, başlık yalan. '100+ ajan', 'şef ajan' ya da 'PM ajan' hiç geçmiyor.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Büyük kısmı var. 4 dakika kuralımız (dxb-cost-gate) 18:24'te söylenen 'alt-ajan önbelleği her yerde 5 dakika' bilgisine dayanıyor. Yeni olan iki ipucu: mola vermeden ya da devretmeden önce, önbellek henüz sıcakken /compact yapmak; geçen testlerin çıktısı bağlamı doldurmasın diye CLAUDE.md'ye sessiz test komutu yazmak.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Tahta satırı yok; inşaat bilgisi</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Bilgi (lider oturumu)</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Makine: kota tasarrufu</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>İzle</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Bizim kuralı doğruluyor; uygulanacak yeni bir parça yok. Önbellek süresini 1 saate çıkarma önerisi 4 dakika kuralı yüzünden geri çekildi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>EK03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>hanakoxbt — 'Karpathy'nin Opus 5.5'i grafiğe çeviren promptu'</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/hanakoxbt/status/2108308634727760066</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Gönderideki tek resim okundu</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>İşi düğümlere bölen, her düğüme kapı, düzeltme ve öğrenme dönüşü koyan uzun bir prompt şablonu.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Başlık yalan. Resmin altında 'Not written or endorsed by Andrej Karpathy' yazıyor; şablonu hesabın sahibi yazmış.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Var. dxb-team2 aynı düzeni zaten kuruyor: plan baş mühendiste, işi yardımcılar yapıyor, her parça doğrulanıyor, Sol kör denetçi, iş devrediliyor.</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>Bizdeki düzenin daha zayıf bir kopyası.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>EK04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>0xkichiro — 'Anthropic mühendisi: %90 kendini geliştiren döngü, ajan grafikleri'</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/0xkichiro/status/2110338483256451241</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>10 dk video; döküm tamamı</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Claude Code ürün müdürü Kat Wu'nun Mayıs 2025 lansman konuşması: Claude Code'un herkese açılması, Claude 4 modelleri, SDK, GitHub Actions.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Başlık yalan. '%90 mühendis', 'döngü' ya da 'grafik' hiç geçmiyor; tek '90' sözü '90 dakika çalıştı' (05:21). Boş terminalden de başlanmıyor; video hızlandırılmış.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Var; bugünkü kurulumumuz bunların ötesinde.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Bir buçuk yıllık lansman videosu, sahte başlıkla paylaşılmış.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>EK05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>hayatomaruu — 'Karpathy: Opus 5.5 harness mühendisliği, kodumun %99'u otomatik'</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/hayatomaruu/status/2110481057418010989</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>30 dk röportaj; döküm tamamı</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Karpathy ile gerçek bir röportaj. Konuları: Software 3.0, doğrulanabilirlik, 'agentic engineering' ve kalite çıtası, spesifikasyon ve veri tasarımının insanda kalması.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Konuşma gerçek, başlık yalan. 'Opus 5.5' demiyor, 'opus 4.7' diyor (11:51). 'Harness' ve '%99' hiç geçmiyor.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Fikirleri bizde var: önce spesifikasyon, kör denetçi, bilgi grafiği.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Bilgi</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Alma</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>İyi bir sohbet; uygulanacak yeni bir teknik yok.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>EK06</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Bonsai 27B (PrismML) — XDA makalesi</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.xda-developers.com/dropped-qwen-and-gemma-for-27b-model-that-runs-smoothly-on-8gb-card/</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Makalenin tamamı</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Qwen3.6 27B'nin 1 bitlik sıkıştırılmış hali: 4,4 GB, 8 GB ekran kartında çalışıyor. Makaledeki ölçümler: matematik 91,7 (tam modelde 95,3), kod 89,6 (95,1), araç kullanma 66 (80).</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Makale gerçek, 10 Ekim 2026 tarihli. Rakamlar üreticinin kendi testlerinden.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Bizde yerel model tezgâhı var (B33). Makinemizdeki ekran kartı 16 GB'lık RTX 5060 Ti; 8 GB sınırımız yok.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>B33 (GPU tezgâhı)</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Hayır</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Makine: ücretsiz yerel özetleme ve sınıflandırma işçisi olabilir</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Araç kullanmada zayıf; ajan işine uymaz</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Kurulum</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>İzle</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>Bize asıl gereken iş araç kullanan ajan; bu model tam orada zayıf. Yerel bir işçi gerekirse tezgâhta denenir.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>EK07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Higgsfield Ads Studio ve Seedance 2.5 — YouTube anlatımı</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=xixxe38ar6g</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>7,5 dk video; döküm tamamı</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Higgsfield'in ücretli reklam aracı. 'Ad multiplier' videodaki kişiyi, ürünü ve ortamı değiştiriyor, açılış cümlesi (hook) ve harekete çağrı (CTA) çeşitliyor. Marka bilgisinden ya da siteden sabit reklam görseli üretiyor.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Araç gerçek; anlatım bir kullanıcının denemesi. Fiyat videoda yok.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Bedava, yerel karşılıkları Excel'de duruyor: W071 (altı ücretsiz video üretici), W076 (MiniMax ile Higgsfield reklamını yeniden üretmek).</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>B43 (stüdyo), B28 (ajans)</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Hayır (stüdyo)</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Gelir: müşteriye 'aylık reklam varyasyonu' hizmeti</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Ücretli (para çıkışı). Kişi değiştirme ve insan görseli helal-tasvir kararınıza (46-49) bağlı.</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Para çıkışı, İslami karar</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>İzle</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>Hizmet fikri iyi; bunu bedava yerel araçlarla, stüdyo sırası geldiğinde yaparız.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>EK08</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Voxyz — iki gönderi (dinamik iş akışı; alt-ajan önbellek süresi)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/Voxyz_ai/status/2109237583704445140 ; https://x.com/Voxyz_ai/status/2109056129884123370</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>13 Ekim'de başka bir oturumda incelendi; bugün resmi dokümanlar okundu</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Claude Code'un Workflow aracı (birçok ajanı bir senaryoyla yönetir) ve alt-ajana 1 saatlik önbellek ayarı (experimental.cacheTtl).</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>İkisi de resmi dokümanda var. '70 hatadan 66'sı bulundu' rakamı iki dokümanda da bulunamadı.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Workflow aracı her oturumda hazır ama holdingde hiç kullanılmadı. Önbellek sorunu bizde 4 dakika kuralıyla zaten çözülmüş.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>4. sıradaki güvenlik taraması</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>İş akışı: o sıra gelince</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>İnşaat: büyük taramalarda hız</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Kota: bir koşu 1.000 ajana kadar çıkabilir</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Sizin sözünüz (iş akışını çalıştırmak)</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>İş akışı: o sırada kullan · Önbellek: yapma</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>Ayrı bir deneme gerekmiyor.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(watch-links): WhatsApp links since 15 Oct 11:40 — sixteen new ones reviewed into a new Excel sheet "Ekim 15-21 linkleri"
Already-reviewed hayatomaruu (15 Oct 11:41) skipped; all sixteen checked absent from every sheet and the records.
Nothing installed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B8fzoxbZeBYmo4EuAvnLgZ
</commit_message>
<xml_diff>
--- a/.planning/research/watch-links/2026-10-08-whatsapp/turbo/Excel-turbo.xlsx
+++ b/.planning/research/watch-links/2026-10-08-whatsapp/turbo/Excel-turbo.xlsx
@@ -14,12 +14,14 @@
     <sheet name="Değişenler" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Yeni eklenenler" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Ekim 9-15 linkleri" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Ekim 15-21 linkleri" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Öncelikli'!$A$1:$Z$64</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Tüm linkler'!$A$1:$Z$89</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Değişenler'!$A$1:$M$72</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Yeni eklenenler'!$A$1:$N$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Ekim 15-21 linkleri'!$A$1:$V$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -59,7 +61,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -91,6 +93,31 @@
         <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -104,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -136,6 +163,27 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -24880,4 +24928,1755 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:V17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="13" max="13"/>
+    <col width="35" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="45" customWidth="1" min="17" max="17"/>
+    <col width="60" customWidth="1" min="18" max="18"/>
+    <col width="40" customWidth="1" min="19" max="19"/>
+    <col width="45" customWidth="1" min="20" max="20"/>
+    <col width="30" customWidth="1" min="21" max="21"/>
+    <col width="25" customWidth="1" min="22" max="22"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="12" t="inlineStr">
+        <is>
+          <t>Tarih</t>
+        </is>
+      </c>
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>Başlık</t>
+        </is>
+      </c>
+      <c r="D1" s="12" t="inlineStr">
+        <is>
+          <t>Ne bu</t>
+        </is>
+      </c>
+      <c r="E1" s="12" t="inlineStr">
+        <is>
+          <t>Tür</t>
+        </is>
+      </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>Holding (0-3)</t>
+        </is>
+      </c>
+      <c r="G1" s="12" t="inlineStr">
+        <is>
+          <t>Holding için neden</t>
+        </is>
+      </c>
+      <c r="H1" s="12" t="inlineStr">
+        <is>
+          <t>Teknoloji (0-3)</t>
+        </is>
+      </c>
+      <c r="I1" s="12" t="inlineStr">
+        <is>
+          <t>Teknolojiye katkısı</t>
+        </is>
+      </c>
+      <c r="J1" s="12" t="inlineStr">
+        <is>
+          <t>Gelir (0-3)</t>
+        </is>
+      </c>
+      <c r="K1" s="12" t="inlineStr">
+        <is>
+          <t>Gelire katkısı</t>
+        </is>
+      </c>
+      <c r="L1" s="12" t="inlineStr">
+        <is>
+          <t>Oturum (0-3)</t>
+        </is>
+      </c>
+      <c r="M1" s="12" t="inlineStr">
+        <is>
+          <t>Oturum için neden</t>
+        </is>
+      </c>
+      <c r="N1" s="12" t="inlineStr">
+        <is>
+          <t>Bizde zaten var mı</t>
+        </is>
+      </c>
+      <c r="O1" s="12" t="inlineStr">
+        <is>
+          <t>Tahta satırı</t>
+        </is>
+      </c>
+      <c r="P1" s="12" t="inlineStr">
+        <is>
+          <t>Öneri</t>
+        </is>
+      </c>
+      <c r="Q1" s="12" t="inlineStr">
+        <is>
+          <t>Not</t>
+        </is>
+      </c>
+      <c r="R1" s="12" t="inlineStr">
+        <is>
+          <t>Uygulama planı</t>
+        </is>
+      </c>
+      <c r="S1" s="12" t="inlineStr">
+        <is>
+          <t>Sizin notunuz</t>
+        </is>
+      </c>
+      <c r="T1" s="12" t="inlineStr">
+        <is>
+          <t>Link(ler)</t>
+        </is>
+      </c>
+      <c r="U1" s="12" t="inlineStr">
+        <is>
+          <t>Neye bakıldı</t>
+        </is>
+      </c>
+      <c r="V1" s="12" t="inlineStr">
+        <is>
+          <t>Okundu mu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>EK09</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>rananjay.ai '20 repo ile Opus 5.5'i hareketli grafik stüdyosuna çevir' listesi — çekirdeği HyperFrames + Remotion + 18 skill/kütüphane</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Instagram'da 9 slaytlık bir liste: Claude Code'un kodla ürün tanıtım videosu, lansman filmi ve animasyonlu anlatım üretmesi için 20 GitHub deposu. Gerçek motorlar ikisi: HyperFrames (HTML/CSS/GSAP → MP4, Apache-2.0, 68.810 yıldız) ve Remotion (React → video, şirket lisansı ister, 65.837 yıldız); geri kalanı bunların üstüne zamanlama, kamera, ses ve 'slop'suz tasarım tarifi veren skill paketleri (ör. product-launch-motion 334, charlie947/motion-graphics-skills 356, howseen-ai/claude-motion-design 613, nateherkai/hyperframes-student-kit 1.933, LottieFiles/motion-design-skill 2.386, remotion-dev/skills 5.464 yıldız) ve web animasyon kütüphaneleri (GSAP, Motion, lottie-web). Son slayt tam listeyi 'MOTION yaz, DM atayım' yemiyle veriyor; ama 20 adın hepsi slaytlarda açık yazılı.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>repo</t>
+        </is>
+      </c>
+      <c r="F2" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Stüdyonun (B43) yazı-grafik-lansman videosu katmanı; motor zaten seçili (HyperFrames, YE03 kararı), liste o motorun üstüne konacak tarifleri gösteriyor.</t>
+        </is>
+      </c>
+      <c r="H2" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>HyperFrames için hazır skill'ler (hyperframes-motion-reel-skill: ritme oturan showreel; product-launch-motion: tek şekil, imleçle sürülen geçiş, 60 fps hareket bulanıklığı; LottieFiles motion-design-skill: zamanlama ve easing ilkeleri) stüdyonun hareketli grafik kalitesini ilk atışta yükseltir; GPU gerektirmez, deterministik.</t>
+        </is>
+      </c>
+      <c r="J2" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>B28 ajans koltuğu için satılabilir ürün: müşteriye kodla üretilmiş SaaS/ürün lansman videosu, açıklayıcı animasyon, sosyal medya kısa grafikleri — GPU beklemeden, düşük maliyetle seri.</t>
+        </is>
+      </c>
+      <c r="L2" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>İnşaat oturumlarına değil, stüdyo işine yarar; yalnız video üretim işi açılınca çekmece açılır.</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Kısmen: HyperFrames stüdyonun aracı olarak alındı (HIS-WORDS-2026-10-15 YE03, tahta sırası #45/B43, telemetri kapalı ölçüldü); Remotion W071'de 'şirket lisansı ister, HyperFrames tercih' diye ayrıldı; W025/W104/W107 aynı yolu işledi. Bu 18 skill paketinin hiçbiri kurulu değil.</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>B43</t>
+        </is>
+      </c>
+      <c r="P2" s="15" t="inlineStr">
+        <is>
+          <t>Dene</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>Remotion ticari kullanımda şirket lisansı ister (3+ kişilik şirkette ücretli) — para çıkışı, onay kapısı; HyperFrames yolu bedava. Paketlerin çoğu MIT; nateherkai kiti ve Barty-Bart 'NOASSERTION' (lisans belirsiz, fikir olarak okunur), klik-anim lisanssız. Hepsini kurmak yerine HyperFrames üstüne en fazla 2-3 tanesi (product-launch-motion, hyperframes-motion-reel-skill, LottieFiles motion-design-skill) tek bir örnek lansman filmiyle denenir; Kanun D: önce taslak. İslami sınır: müzik/ses seçimi stüdyonun mevcut kuralına tabi.</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>20 deponun hepsi kurulmaz; HyperFrames üstüne en iyi 2-3 tarif paketi (product-launch-motion gibi) EK16 denemesinde seçilir.</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr"/>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/p/DeRvxD6gDCu/</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>9 slaytın hepsi okundu (carousel.py); 20 deponun 20'si gh api ile doğrulandı (yıldız, son itme, lisans).</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr">
+        <is>
+          <t>evet — slaytlar ve her depo gh api ile; README'ler okunmadı, yalnız açıklamalar</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>EK10</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>REA — Reverse Engineer Anything (morluto/rea): ajanla kapalı kaynak programın bir özelliğini çözüp kendi ürününe yazdırma</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>HQ NET'in Türkçe videosu REA skill'ini deniyor: ajan Ghidra/Hopper/IDA, JADX gibi araçlarla ikili dosyanın fonksiyon referanslarına iner, mantığı anlar ve istenen dilde benzerini yazar. Yaratıcı iki örnek gösteriyor: OBS'in mikrofon filtrelerini canlı çalışan mini bir uygulamaya çevirmek ve Windows Fotoğraflar'ın 'arka planı kaldır' özelliğini kendi ekran-alıntısı aracına sağ tık menüsüyle eklemek (~40 dakika sürdü, çalıştığı ekranda görüldü). Depo gerçek: morluto/rea, MIT, 352.811 yıldız, 2026-04-14'te açılmış, bugün güncellenmiş; npx rea-agents setup ile Claude Code'a MCP sunucusu + iş akışı skill'i kurar, analiz yerelde koşar ve her sonucun kanıtını verir.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>araç</t>
+        </is>
+      </c>
+      <c r="F3" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Holdingin makinesi kendi kodumuz ve açık kaynak üstüne kurulu; kapalı bir programın ikili dosyasını sökmeye ihtiyaç duyduğu bir iş bugün tahtada yok. Değeri dar: bir rakibin/aracın davranışını incelemek.</t>
+        </is>
+      </c>
+      <c r="H3" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Bir Electron/JS uygulamasının (ör. bir rakip masaüstü aracı) mimarisini kanıtla çıkarmak dxb-rival-intel'e bir el olabilir; ama web tarafı zaten scrapling/playwright ile okunuyor.</t>
+        </is>
+      </c>
+      <c r="J3" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Doğrudan gelir yolu yok; 'beğendiğin özelliği kendi ürününe koy' hızlandırıcısı olarak dolaylı. Kapalı yazılımın kodunu kopyalayıp satmak telif riskidir.</t>
+        </is>
+      </c>
+      <c r="L3" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>Oturumlara düzenli fayda yok; MCP + 170 araç açılış bağlamını şişirir. Gerekirse aicodeking/leanrea (8 KB, MCP'siz, 1.226 yıldız) daha hafif yol.</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Yok (repoda REA/reverse engineer anything izi bulunmadı).</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+      <c r="P3" s="16" t="inlineStr">
+        <is>
+          <t>İzle</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>Hukuki ve ahlaki sınır: kapalı kaynak yazılımı tersine mühendislikle kopyalamak lisans sözleşmesini ve telifi çiğneyebilir; videodaki yaratıcı da 'yasal kullanın' diyor. Holdingde kullanım ancak anlamak/ilham almak için, kod kopyalamadan olur — bu, kul hakkı yönünden de gerekli. Kurulum Hopper/Ghidra/JDK indirir; bir iş gerektirene kadar kurulmaz. Taklit depolar var (README 'resmî kaynak yalnız morluto/rea, rea.tools, rea-agents npm' diye uyarıyor).</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>Kurulmaz. Kapalı yazılımı tersine mühendislikle kopyalamak lisans ve kul hakkı sınırına takılır; yalnız anlamak için izlenir.</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>Linkini değil, dizüstündeki videonun telefonla çekilmiş fotoğrafını attınız: "Yazılımları Klonlayan Yeni REA Skill'ini Denedim" (HQ NET).</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=vsFS1Ei79Qs</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>a) transkriptin tamamı okundu (10 dk); b/c yapılmadı — demo anlatımla yeterince açık, araç gh api + README ile doğrulandı.</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr">
+        <is>
+          <t>evet — transkript tam, README'nin kurulum ve çalışma bölümü okundu</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>EK11</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Mert Durmazer: açık kaynak Umami'yi ekran görüntüsünden 13 dakikada kopyalayıp 'yapay zekâdan gelen trafiği ölçen' niş ürüne çevirmek ve pazarlamasını Claude'a yaptırmak</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Video REA'yı (82 bin yıldız dediği andaki sayı) hedef almıyor, aslında ona gerek olmadığını söylüyor: MIT lisanslı Umami web analitiğinin herkese açık demosundan 5 ekran görüntüsü verip Opus 5.5'e tek istemle kopyasını kurduruyor (13 dk), sonra 'yapay zekâ asistanlarının (ChatGPT, Perplexity) siteye gönderdiği ziyaretçiyi ayrı kanal olarak gösteren' tek bir yeni özellikle farklılaştırıyor (10 dk, API fiyatıyla 3,32 $). Ardından konumlandırma, landing page, ilk 30 gün müşteri planı, Product Hunt sloganı ve isim/alan adı araştırmasını Claude'a yaptırıyor (5 dk, 1,62 $); 'uydurma sayı, sahte yorum yok' kuralı koyuyor. Tezi: kod ucuzladı, değeri kime hangi cümleyle satacağın belirler; tutmuş bir piyasayı (rakipler aylık 29-99 $) daha dar bir kitleye (ör. klinikler) götür.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>gelir fikri</t>
+        </is>
+      </c>
+      <c r="F4" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Yöntemi holdingin gelir makinesine birebir oturuyor: kanıtlanmış açık kaynak ürünü al → tek farklılaştırıcı özellik → dar kitle → Claude ile pazarlama. Holding az insanla çok ürün çıkarabilen bir fabrika.</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Yeni araç yok; 'ekran görüntüsünden klon + tek fark' akışı mevcut inşaat yöntemimizle yapılabilir.</t>
+        </is>
+      </c>
+      <c r="J4" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Somut fikir: 'yapay zekâ görünürlüğü' analitiği (GEO/AEO) — W073 AI SEO ajansı fikriyle aynı pazar; holdingin müşterilerine (ör. Türkiye'deki klinik, e-ticaret) aylık abonelik ya da ajans hizmetinin ölçüm ayağı olarak satılabilir. Umami MIT olduğu için meşru temel. Önce talep sınaması gerekir.</t>
+        </is>
+      </c>
+      <c r="L4" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Oturumlara yeni bir şey getirmiyor.</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>Kısmen: W073 (Searchmaxxed AI SEO/GEO ajansı) ve W094 (aynı yaratıcının AgencyOS videosu) tahtadaki link kayıtlarında; yapay zekâ trafiği ölçen ürün yok.</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>B17</t>
+        </is>
+      </c>
+      <c r="P4" s="14" t="inlineStr">
+        <is>
+          <t>Araştır</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>Lisans: yalnız MIT/Apache gibi izin veren açık kaynak üzerine kurulur; kapalı ürünü kopyalamak telif ihlali (yaratıcı da söylüyor). Videodaki sayılar (13 dk, 3,32 $) yaratıcının beyanı, ölçülmedi. Yapay zekâ yönlendiren bilgisi (referrer) çoğu uygulamada gelmez — ürün eksik sayar, yaratıcı bunu dürüstçe söylüyor; ürünün değeri bu ölçüm sınırına bağlı. Aynı pazarda rakipler var (aylık 29-99 $). Para çıkışı (alan adı, reklam) onay kapısında.</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>'Yapay zekâ asistanlarından gelen ziyaretçiyi ölçen analitik' niş ürün fikri, 16 gelir yapısı raporuna (B17) bir satır olarak girer; yalnız MIT/Apache tabanla.</t>
+        </is>
+      </c>
+      <c r="S4" s="2" t="inlineStr">
+        <is>
+          <t>Linkini değil, dizüstündeki videonun telefonla çekilmiş fotoğrafını attınız: "Viral Olan 'Her Şeyi Tersine Mühendislik' Skill'ini Test Ettim" (Mert Durmazer).</t>
+        </is>
+      </c>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ZJj4_egB30Q</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>a) transkript tamamı okundu — 3:50-10:00 arası konuşma-metin dönüşümünde bozuk ('bir hızlı' tekrarı); b) o aralık 9 kareyle görüldü (kopya adımı, özellik kontrol listesi, '3 — Daha iyi ürün' slaytı, yönlendiren testi neden başarısız oldu ekranı). c) yapılmadı.</t>
+        </is>
+      </c>
+      <c r="V4" s="2" t="inlineStr">
+        <is>
+          <t>kısmen — transkriptin 6 dakikası bozuk, o aralık yalnız karelerle görüldü; ürünün kendisi (Sightflow/Siteli) yayımlanmamış, denenemedi</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>EK12</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Is Agentic (is-agentic.com) — bir sitenin yapay zekâ ajanlarına ne kadar hazır olduğunu 0-100 puanlayan tarayıcı</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Vercel'in yayımladığı, kontrolleri Ora'nın koştuğu ücretsiz bir tarama aracı: bir alan adı girilir (ya da npx is-agentic &lt;alan&gt;), ajanların siteyi bulup, erişip, anlayıp kullanabilmesine göre puan verir. Kontroller: botlara kapalı mı, JavaScript'siz içerik, Markdown içerik müzakeresi, llms.txt/ajan talimatı, OpenAPI şeması, JSON hata yanıtları, ajana uygun 404, OAuth, MCP yüzeyi vb.; zorunlu kontroller 80, önerilenler 20 puan, en çok 5 bonus. Her rapor eksikler için 'iyileştirme istemi' üretir. Örnek: wordpress.com 42, apple.com 51, vercel.com 95.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>araç</t>
+        </is>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Holdingin satacağı ürün ve markaların sitelerinin ajanlar (ChatGPT, Claude, Perplexity alışveriş/araştırma ajanları) tarafından bulunup kullanılması gelirin yeni kapısı; bu araç ölçüyü bedava veriyor.</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Holdingin kendi kamuya açık sitelerinin (stüdyo, ajans, ürün sayfaları) yayın öncesi kontrol listesine bir satır: is-agentic puanı ve önerdiği düzeltmeler (llms.txt, Markdown yanıt, JSON hatalar). Kendi kodumuza bir şey eklemiyor.</t>
+        </is>
+      </c>
+      <c r="J5" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Ajans hizmeti olarak satılabilir: müşterinin sitesini tara → 'ajan hazırlığı' denetim raporu → düzeltme paketi; W073 AI SEO/GEO ajansı ve EK11'in yapay zekâ trafiği ölçümüyle aynı pakette. Araç bedava, emek bizim — düşük maliyetli giriş teklifi.</t>
+        </is>
+      </c>
+      <c r="L5" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>İnşaat oturumlarına katkısı yok.</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Yok; repoda is-agentic/agent readiness izi bulunmadı (llms.txt yalnız fal.ai fiyat okumada geçiyor).</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>B28 / B17</t>
+        </is>
+      </c>
+      <c r="P5" s="15" t="inlineStr">
+        <is>
+          <t>Dene</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>Ücretsiz, hesap ve anahtar gerekmez; taranan alan adı Vercel/Ora'ya gider (müşteri sitesi taranacaksa müşterinin kamuya açık sitesi olduğu için sorun yok). Puan bir özet; değer tek tek kontrollerde. Holdingin henüz kamuya açık bir sitesi olup olmadığı bu okumada ölçülmedi. Satış paketine girerse önce bir müşteri sitesinde örnek rapor hazırlanır.</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>is-agentic.com ile önce kendi müşteri sayfamız (klinik) taranır; puan ve eksikler ajansın 'sitenizi yapay zekâ ajanlarına hazırlıyoruz' hizmet kalemine malzeme olur.</t>
+        </is>
+      </c>
+      <c r="S5" s="2" t="inlineStr"/>
+      <c r="T5" s="2" t="inlineStr">
+        <is>
+          <t>https://is-agentic.com/</t>
+        </is>
+      </c>
+      <c r="U5" s="2" t="inlineStr">
+        <is>
+          <t>Video yok; ana sayfa, wordpress.com tarama raporu ve Methodology sayfası fetch.py ile okundu.</t>
+        </is>
+      </c>
+      <c r="V5" s="2" t="inlineStr">
+        <is>
+          <t>evet — ana sayfa, bir örnek rapor, metodoloji</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>EK13</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic'ten Gagan Bhat'ın 'Claude Managed Agents' konuşması — X'te '250-750 bin $ maaşlı mühendis harness kurmayı öğretiyor' diye pazarlanmış</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>X gönderisi (shikamarutsai) 12 dakikalık bir videoyu 'Anthropic bu mühendisi 250-750 bin $'a aldı, sıfırdan çoklu-ajan harness kurmayı 5 adımda gösteriyor' diye sunuyor; maaş iddiası ve 5 adım videoda yok, uydurma kanca. Videonun kendisi: Anthropic'ten Gagan Bhat, ajan arayüzlerinin evrimini anlatıyor — Messages API → Claude Agent SDK (döngü, bağlam, araçlar sende) → Claude Managed Agents (döngü Anthropic sunucusunda koşar; ajan, ortam ve oturum üç kaynak; beyin ile sandbox ayrı, sandbox gerekince açılır; oturum bulutta kalıcı, laptop kapansa da sürer; olaylarla yönlendirilir). Ek özellikler: alt-ajanlar, hafıza, 'dreaming' (geçmiş transkriptlerden skill ve hafıza üretme), outcomes (çıktıyı yineleyerek iyileştirme), vault (kimlik bilgisi kasası), webhook, izin politikası, zamanlanmış/tetiklenen ajanlar. Atölye kodu anthropics/cwc-workshops/ship-your-first-managed-agent (SRE ajanı örneği).</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>eğitim</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Holdingin 7/24 kendi kendine çalışma vaadinin altyapı sorusuna doğrudan dokunuyor: Hermes'in sunucusu silindi (B09/B11), gece işçisi ve uzun koşu bir sunucu ister; Managed Agents sunucu tutmadan bulutta koşan, kaldığı yerden süren, zamanlanabilen ajan sunuyor.</t>
+        </is>
+      </c>
+      <c r="H6" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Üç fikir doğrudan makineye: (1) beyin ile ellerin ayrılması ve oturumun olay günlüğünden devam etmesi — Hamza'nın uzun işleri için; (2) 'dreaming' — C39'daki şirket doktoru fikrinin (tüm koşulardan tekrar eden kusuru bulup onarım önermek) Anthropic'teki karşılığı; (3) zamanlanmış/tetiklenen ajanlar — B11 gece işinin sunucusuz yolu. Hepsi önce ölçülmeli: fiyat, veri yeri, mevcut çalışma zamanımızla (Agent SDK) çakışma.</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Dolaylı: müşteriye sunulacak ajan ürünlerini (ör. ajansın müşteri ajanları) sunucu yönetmeden barındırma yolu; doğrudan gelir yolu değil.</t>
+        </is>
+      </c>
+      <c r="L6" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>İnşaat oturumlarına değil, holdingin çalışma zamanına yarar; cwc-workshops'taki 'agents-that-remember', 'eval-driven-agent-development', 'rightmodel' klasörleri ileride B51 model mimarisi için okunabilir.</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>Kısmen: Agent SDK holdingin çalışma zamanında kullanılıyor (B65 Agent SDK sonucu); 'Managed Agents' tahtada B42 satırında ve b64 araştırma notlarında (r-multiagent.md, v2v3-mods-anthropic.md) geçiyor; dreaming fikri C39'da adıyla duruyor. Managed Agents'a geçiş kararı yok.</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>B09 / B11</t>
+        </is>
+      </c>
+      <c r="P6" s="14" t="inlineStr">
+        <is>
+          <t>Araştır</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>Gönderinin maaş ve '5 adım' iddiası videoda yok — kanca. Managed Agents ücretli bir API ürünü (para çıkışı, onay kapısı) ve ham sağlayıcı anahtarı ister; STACK.md 'ikinci iş çalışma zamanı yok, ham sağlayıcı anahtarı yok' diyor — benimsemek bir mimari karar, önce STACK.md ve B51 ile çatışması ölçülür. Veriler Anthropic bulutunda kalır.</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>Managed Agents yalnız B09/B11 (Hermes'in beyni) kararında bir seçenek olarak okunur; STACK.md 'ikinci iş çalışma zamanı yok, ham anahtar yok' dediği için şimdi benimsenmez.</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr"/>
+      <c r="T6" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/shikamarutsai/status/2110817965658571181</t>
+        </is>
+      </c>
+      <c r="U6" s="2" t="inlineStr">
+        <is>
+          <t>a) transkriptin tamamı okundu (12 dk); b) 7 kare görüldü (konuşmacı adı ve unvanı, mimari slaytları); anthropics/cwc-workshops deposunun klasörleri gh api ile doğrulandı. c) yapılmadı.</t>
+        </is>
+      </c>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
+          <t>evet — video tam transkript + kareler; gönderinin altındaki 'Opus 5.5 harness rehberi' alıntısı (beamnxw) okunmadı, pazarlama zinciri</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>EK14</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>TasteSkill v2 (Leonxlnx/taste-skill, 'design-taste-frontend') — sayfayı üç genişlikte açıp yapay zekâ sitesi izlerini listeleyen tasarım skill'i</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Vox'un 15 Ekim gönderisi (768 beğeni, 46.947 görüntülenme) bulundu: TasteSkill v2'yi kurup Opus 5.5'e sitenin 'check-up'ını yaptırmayı öneriyor — inspect.mjs sayfayı masaüstü/tablet/telefon genişliğinde gerçek tarayıcıda açar, 'AI sitesi' işaretlerini (başlık üstü küçük büyük harfli satır, 01/02/03 bölüm numarası, gövdede monospace, hover'sız gradyan/gölge, krem+terakota ya da mor-indigo, 4'ten az gerçek resim) sayfa, genişlik ve öğe adıyla listeler; gönderi hazır bir 'kod değiştirme, önce listeyi göster' istemi veriyor ve dürüstçe kör testte farkın neredeyse sıfır (7,7'ye 7,8) olduğunu söylüyor. Skill gerçek: MIT, 100.155 yıldız, v2.1.4 (2026-10-20); v2 247 seçilmiş siteden derlenmiş, 20 yön arasından seçer, açık arşivlerden kaynaklı gerçek görsel kullanır, tarayıcıda kontrol edip üç tura kadar düzeltir; v2.1 panolar ve uygulama ekranları için ayrı yol ekledi.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>araç</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>CEO'nun gördüğü her yüzey ve holdingin satacağı her sayfa Ferrari çıtasında olmalı; 'yapay zekâ yapımı görünme' bu çıtanın en sık düştüğü yer. Üç genişlikte gerçek tarayıcı denetimi B03-bis'in (giriş yapılmış CEO yüzeylerinin gerçek tarayıcı göz kontrolü) yanında ikinci bir göz.</t>
+        </is>
+      </c>
+      <c r="H7" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>inspect.mjs yayın öncesi otomatik 'slop' denetimi olarak dxb-surface kapısının yanında koşturulabilir; v2.1 pano kuralları (sessiz paneller, hizalı rakamlar, rengi veriye harcamak, telefonda katlanan menü) CEO panosuna doğrudan uyar. Ölçülmesi gereken: kendi tasarım hükümlerimizle (C-hibrit yön, 17 Temmuz kart kuralları) çelişip çelişmediği.</t>
+        </is>
+      </c>
+      <c r="J7" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Ajansın müşteriye yaptığı landing page'lerin kalitesini yükseltir ve 'site check-up' küçük bir hizmet olarak satılabilir; tek başına gelir yolu değil.</t>
+        </is>
+      </c>
+      <c r="L7" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Yüzey işinde oturuma hazır bir tarayıcı denetçisi verir; ama tam bir yapım 30-45 dk ve birkaç yüz bin jeton yer — yalnız denetim (inspect) modu ucuz kullanım.</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>Kısmen: taste-skill eklentisi kurulu ama kapalı (~/.claude/plugins/marketplaces/taste-skill, son güncelleme 2026-07-23 — v2 öncesi, eski); 2026-09-19 açılış planında 'Faz 8 tasarım işi başlayınca çekmece açılır' kararıyla dolapta; rows-D.md'de tasarım paketlerinin CEO kararı 'adı konmuş çatışma, onda' diye açık.</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>B03-bis / B32</t>
+        </is>
+      </c>
+      <c r="P7" s="17" t="inlineStr">
+        <is>
+          <t>Kur</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>Eklentiyi açmak/güncellemek CEO'nun açık 'tasarım paketleri' kararına dokunur — önce ona tek satır sorulur (kapatma/açma öncesi sor hatırası). Kendi kör testlerinde fark neredeyse yok (7,7'ye 7,8): yapım aracı olarak değil, denetim listesi olarak değerli. Node 22+ ve Chrome ister, anahtar istemez; görsel bulmak için ağa çıkar, açık arşiv görsellerinin lisansı skill'in kredi dosyasıyla izlenir. 2.1.4'te tarayıcı profili silme hatası düzeltildi — eski sürüm kullanılmamalı. Görsel kaynaklarında haram içerik süzgeci holdingin kuralıyla ayrıca uygulanır.</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>Eklentinin eski v1 kopyası kaldırılıp en yeni sürüm kurulur (sizin sözünüz, 21 Ekim); eklenti yine kapalı durur. inspect.mjs ile sayfayı üç genişlikte açan 'yapay zekâ sitesi izi' denetimi, B03-bis göz kontrolüne ve müşteri sitelerinin teslim öncesi kontrolüne liste olarak eklenir.</t>
+        </is>
+      </c>
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>Linksiz, telefondan ekran görüntüsü attınız: Vox (@Voxyz_ai) TasteSkill v2 önerisi; gönderi ve aracın kendisi bulundu.</t>
+        </is>
+      </c>
+      <c r="T7" s="2" t="inlineStr"/>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>Video yok; Vox'un gönderisi opencli ile bulundu ve okundu (alıntıladığı önceki gönderi dahil); depo gh api, README, CHANGELOG ve son commit'lerle okundu.</t>
+        </is>
+      </c>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>evet — gönderi, README, CHANGELOG 2.1.2-2.1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>EK15</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Claude Code /loop ile sayfa sayfa SEO denetimi</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Bir pazarlamacı, Claude Code'da /loop komutuyla web sitesini sayfa sayfa SEO açısından (teknik, metin, izleme) analiz ettirip her sayfa için değişiklik günlüğünü PDF olarak kaydettirmeyi, sayfayı 'bitti' diye işaretletip sıradakine geçirmeyi öneriyor. İddia: tüm siteye tek seferde bakmak yerine sayfa sayfa çalışmak daha iyi sonuç verir. Gösterilen tek şey terminale yazılan bir istem; araç, ölçüm ya da sonuç yok.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>strateji</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Fikir doğru ama sıradan: uzun bir listeyi parça parça, her parçanın kaydını tutarak işlemek. Holdingin kendi sitesi ve ajans müşterileri için bir hizmet kalıbı olabilir; yeni bir yetenek getirmiyor.</t>
+        </is>
+      </c>
+      <c r="H8" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>/loop zaten Claude Code'da yerleşik bir beceri ve bu oturumda listede duruyor; 'liste → bir öğe → kayıt → işaretle → sıradaki' kalıbı bizim iş kuyruğumuzun bildiği bir şey.</t>
+        </is>
+      </c>
+      <c r="J8" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>B28 ajans koltuğunda müşteri sitelerine sayfa başı SEO denetimi + PDF rapor küçük bir hizmet kalemi olabilir; ancak videoda kalite ya da sonuç kanıtı yok, değeri denemeden bilinmez.</t>
+        </is>
+      </c>
+      <c r="L8" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>/loop'u uzun sıralı işlerde kullanma hatırlatması; yeni bir şey öğretmiyor.</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>Evet — /loop Claude Code'da yerleşik (bu oturumun beceri listesinde 'loop'); dxb-research araştırma tarafını taşıyor. Holdingin SEO hizmeti için ayrı bir satır yok.</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>B28 (reklam/ajans işi) — ileride ajans hizmet kalemi olarak</t>
+        </is>
+      </c>
+      <c r="P8" s="18" t="inlineStr">
+        <is>
+          <t>Gerek yok</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>Para çıkışı yok, risk yok. Videoda 'birkaç dakika bekle, tekrar et' denen döngü, sayfa listesi bitince durdurulmazsa boşuna kota yakar; kullanılırsa döngüye bitiş koşulu yazılmalı. CEO notu boş.</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="inlineStr"/>
+      <c r="S8" s="2" t="inlineStr"/>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/reel/DehmfSekvuX/</t>
+        </is>
+      </c>
+      <c r="U8" s="2" t="inlineStr">
+        <is>
+          <t>a) transkriptin tamamı okundu (76 sn); b) 4 kare (3, 12, 30, 60. sn) — ekranda yalnız /loop istemi yazılıyor; c) gerekmedi</t>
+        </is>
+      </c>
+      <c r="V8" s="2" t="inlineStr">
+        <is>
+          <t>evet — videonun tamamı transkriptten, ekrandaki istem karelerden okundu</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>EK16</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Claude ile kodla yapılmış 20 video efekti (Remotion tarzı kompozisyonlar)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Türk içerik üreticisi @aykutucesai, tek bir masa başı çekimine Claude'a yazdırılan kodla 20 efekt uyguluyor: orbit, screen wall, UI world, frame break, digital zoom, phone mockup, checklist, headline wall, zoom-through cut, chart grow, pull-back reveal, green screen, paper cut, doodle boil, vertigo, cover story, glass type, kinetic captions, freeze frame, speed ramp. Sondaki kod ekranında `&lt;Sequence from=…&gt;`, `&lt;OrbitCards&gt;`, `&lt;FrameBreak&gt;`, `&lt;GlassType&gt;`, `&lt;SpeedRamp&gt;`, `render("20-efekt.mp4")` görünüyor — React tabanlı video-as-code (Remotion'un Sequence bileşeni) ya da HyperFrames benzeri bir yığın; araç adı videoda söylenmiyor. İddia: efekt adını aynen yazarsan Claude ne istediğini anlıyor.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>eğitim</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>Medya stüdyosu ve reklam işi için doğrudan kullanılır bir efekt sözlüğü: 20 adlandırılmış, kodla üretilebilen kurgu kalıbı. Efektlerin hepsi gerçek ve işler görünüyor (green screen arka plan değişimi, kinetic captions, chart grow, cover story vb.), yani boş bir iddia değil.</t>
+        </is>
+      </c>
+      <c r="H9" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Stüdyonun HyperFrames hattına (CEO kararı YE03, #45, B43) hazır bir efekt kataloğu: her ad bir şablon/bileşen olarak yazılıp kütüphaneye konursa ajanlar 'doodle boil ekle' gibi tek sözle kurgu yapabilir. Yeni araç kurmak gerekmiyor.</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Kısa reklam/Reels klipleri için kurgu programı olmadan, düşük maliyetle tekrar üretilebilir efektler — B28 ajans koltuğu ve B43 stüdyo sekmesindeki müşteri işlerinin değerini artırır; aynı kalıp holdingin kendi içerik kanalları için de geçerli.</t>
+        </is>
+      </c>
+      <c r="L9" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Oturumların değil stüdyonun işi; oturuma etkisi, efekt adlarının kurgu isteminde ortak dil olması.</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>Kısmen — HyperFrames stüdyonun aracı olarak seçildi (HIS-WORDS-2026-10-15 YE03; ORDER.md #45, B43); Remotion'ın şirket lisansı ücretli olduğu için yerine HyperFrames alındı (20261014-88-link okuması). 20 efektlik bir şablon kütüphanesi kayıtlarda görünmedi.</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>B43</t>
+        </is>
+      </c>
+      <c r="P9" s="15" t="inlineStr">
+        <is>
+          <t>Dene</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>Önerilen ilk deneme: stüdyo, 20 efektten 3-4'ünü (kinetic captions, green screen, chart grow, cover story) HyperFrames'te kendi çekimimizle üretsin ve sonucu CEO'nun gözüne koysun. Videodaki kod Remotion söz dizimine benziyor; Remotion'ın ticari kullanımı şirketler için ücretli lisans ister — aynı efektler HyperFrames'te yazılmalı. Green screen arka planları ve doodle'larda haram imge olmamasına dikkat; içeriğe dini konu girerse İslami editoryal kontrol (B43) geçerli. CEO notu boş.</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>Videodaki 20 efektten 3-4'ü (kinetic captions, green screen, chart grow, cover story) HyperFrames'te kendi çekimimizle üretilip gözünüze konur. EK09'daki repo listesi de bu denemenin malzemesi.</t>
+        </is>
+      </c>
+      <c r="S9" s="2" t="inlineStr"/>
+      <c r="T9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/reel/DejsqKlT71p/</t>
+        </is>
+      </c>
+      <c r="U9" s="2" t="inlineStr">
+        <is>
+          <t>a) transkriptin tamamı okundu (98 sn); b) 12 seçili kare; c) watchall ile tamamı — 9 sayfanın hepsi okundu, 20 efektin her biri ekranda görüldü</t>
+        </is>
+      </c>
+      <c r="V9" s="2" t="inlineStr">
+        <is>
+          <t>evet — ses, seçili kareler ve videonun tamamı kare kare görüldü</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>EK17</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>'Andrew Ng'in Graph Engineering kursu' — aslında DeepLearning.AI'ın 'AI Agents in LangGraph' kısa kursunun yeniden yüklemesi</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Gönderi, Andrew Ng'in 'tek ajandan tam otomasyona' 2 saatlik yeni bir Graph Engineering kursu yayımladığını, bölümlerin 'ilk ajan → döngü mühendisliği → graf mühendisliği → kendini yeniden yazan ajanlar' diye ilerlediğini söylüyor. Video (1 sa 52 dk) karelerden okununca: Andrew Ng'in tanıtımı, LangChain/Tavily teşekkür sayfası, 'AI Agents in LangGraph — Persistence and Streaming' başlık sayfası, Jupyter'de LangGraph kodu, 'Reflection' ve 'Supervisor → Agent 1/2/3' çok ajanlı şema; köşede '@GraphsCourse' damgası ve sonradan eklenmiş altyazılar. Yani bu, DeepLearning.AI'ın LangChain ile yaptığı, ücretsiz ve yeni olmayan LangGraph kısa kursunun başka bir hesapça kesilip yeni adla yeniden yüklenmesi. Aramada 'graph engineering' adlı bir Ng kursu bulunamadı; 'döngüden grafa' sıralamasının Ng'in değil yorumcuların kurgusu olduğu yazılıyor.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>eğitim</t>
+        </is>
+      </c>
+      <c r="F10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>İçerik gerçek ama eski ve bizim yolumuzun dışında: LangGraph ile ajan kurmayı öğretiyor. Holdingin yığını LangChain/LangGraph'ı orkestrasyon çekirdeği olarak açıkça reddediyor (STACK.md: Claude Agent SDK zaten araç döngüsü, alt-ajan, MCP ve oturumları taşıyor). Gönderideki 'Andrew Ng yeni kurs yayımladı, 2026' çerçevesi yanıltıcı.</t>
+        </is>
+      </c>
+      <c r="H10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Kalıpların kendisi (reflection, kalıcılık/durum kaydı, supervisor-işçi) bizde zaten Hamza yönlendiricisi, kuyruk ve kalite kapısında var; LangGraph kodu doğrudan kullanılmaz.</t>
+        </is>
+      </c>
+      <c r="J10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Gelir yolu yok.</t>
+        </is>
+      </c>
+      <c r="L10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Oturumların bilmediği bir şey öğretmiyor; ikinci bir ajan çatısı kurmak STACK.md'de yasak ('no second agent framework').</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>Evet — eşdeğer kalıplar Claude Agent SDK + Hamza orkestratöründe; LangGraph STACK.md'de reddedilenler listesinde.</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>Yok</t>
+        </is>
+      </c>
+      <c r="P10" s="18" t="inlineStr">
+        <is>
+          <t>Gerek yok</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>Yeniden yüklenmiş içerik: asıl sahibi DeepLearning.AI/LangChain; telif açısından bu kopyayı paylaşmak ya da kullanmak gereksiz, asıl kurs zaten ücretsiz. Lider tam transkript isterse: bash "/home/dxb/DxB Global OS/.claude/skills/dxb-watch-links/watch.sh" $J EK17 https://x.com/Dhruvkumar16797/status/2111766839516917979 (video akışı indi, ses akışı DOWNLOAD_FAILED ile düştü). CEO notu boş.</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="inlineStr"/>
+      <c r="T10" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/Dhruvkumar16797/status/2111766839516917979</t>
+        </is>
+      </c>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>b) 12 kare (bölüm zamanları dahil: 5, 60, 554, 1200, 1991, 3000, 3766, 4500, 5415, 6000, 6545 sn) okundu; a) transkript alınamadı — 112 dakikalık sesin yazıya dökülmesi bu okuyucunun 4 dakikalık sınırını aştı; arka planda sürdürülen iş sonunda DOWNLOAD_FAILED verdi (ses akışı inmedi); c) yapılmadı</t>
+        </is>
+      </c>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>kısmen — gönderi ve yanıtlar okundu, kurs kimliği karelerden ve aramayla belirlendi; sesin tamamı dinlenmedi</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>EK18</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic'in resmi claude-security eklentisi (çok ajanlı güvenlik taraması)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Gönderi, Anthropic'in resmi pazar yerindeki claude-security eklentisini kurup tüm depoyu taramayı öneriyor. Eklentinin kendi README'si doğruluyor: ajanlar mimariyi ve tehdit modelini çıkarıp bileşen bileşen açık arıyor, her aday bulgu onu çürütmekle görevli bağımsız doğrulayıcılara gidiyor ve yalnız doğrulamayı geçen bulgu rapora giriyor; doğrulama sayımı kodda hesaplanıyor. Rapor MD + JSONL + SARIF olarak depoda zaman damgalı bir klasöre yazılıyor; 'Suggest patches' her bulgu için ayrı, test edilmiş ama uygulanmamış bir yama dosyası üretiyor. Gönderideki 'üç ajandan ikisi onaylarsa' ifadesi README'de 'iki doğrulayıcı derecelendirdikten sonra' şeklinde, tam sayı yazılmıyor.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>araç</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Holding sırlar, şirket veritabanı, ödeme ve kimlik adımları taşıyan bir sistem; kendi kodumuzda saldırılabilir yolları bağımsız doğrulamayla bulan resmi bir araç makinenin sağlamlığını doğrudan artırır. Yanıtlardaki bir kullanıcı ilk taramada migration dosyasında unutulmuş canlı servis anahtarı bulduğunu yazıyor — tam bizim 'sırlar asla depoya girmez' sınırımızın denetimi.</t>
+        </is>
+      </c>
+      <c r="H11" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Kod tabanında sürekli bir güvenlik ölçüsü: tüm depo taraması + her dalın diff taraması, SARIF ile makinece okunabilir çıktı, bulgu kimlikleri taramadan taramaya sabit (yeni/bilinen ayrımı). dxb-verify bataryasına bir güvenlik ayağı olarak bağlanabilir.</t>
+        </is>
+      </c>
+      <c r="J11" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Doğrudan gelir yok; dolaylı olarak, müşteri ve ödeme entegrasyonları (B05) açılmadan önce güvenlik zemini sağlar.</t>
+        </is>
+      </c>
+      <c r="L11" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>İnşaat oturumlarına resmi, doğrulamalı bir güvenlik denetimi ekler; şu an elimizdeki yerleşik /security-review yalnız bekleyen değişikliğe bakıyor, tüm depoyu ve tehdit modelini kapsamıyor.</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>Hayır — eklenti makinedeki claude-plugins-official pazar yerinde duruyor (~/.claude/plugins/marketplaces/claude-plugins-official/plugins/claude-security) ama kurulu/etkin eklentiler listesinde yok. Yerleşik /security-review becerisi var (yalnız bekleyen değişiklik).</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>B51 / B42</t>
+        </is>
+      </c>
+      <c r="P11" s="15" t="inlineStr">
+        <is>
+          <t>Dene</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>Maliyet: büyük depoda onlarca dakikadan birkaç saate kadar sürüyor ve kotanın ciddi kısmını yiyor (yanıttaki kullanıcı: 'haftalık kullanımımın ciddi kısmı'); para çıkışı değil ama kota harcaması — ilk deneme dar bir kapsamla (ör. packages/ ya da bir dalın diff'i) ve medium/high effort ile yapılmalı. Python ≥3.9 ve Dynamic workflows açık olmalı. Lisans: Anthropic'e ait, yalnız iç kullanım — dağıtılamaz, değiştirilmiş hali paylaşılamaz (B27'deki belge becerileri gibi; kopyalanıp depoya konmaz). Çıktı klasörü kendi .gitignore'unu taşıyor. Tarama depodaki CLAUDE.md ve hook'ları normal oturum gibi uygular; dxb-cost-gate gibi kancalar uzun koşuyu kesebilir — koşu lider oturumda yapılmalı. CEO notu boş.</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic'in resmi claude-security eklentisiyle depoya dar kapsamlı bir güvenlik taraması: önce packages/ ve scripts/, sonra bütün depo. Acele sebebi ölçüldü: holdingin GitHub deposu herkese açık (gh repo view → PUBLIC), sızmış anahtar ya da açık varsa dünya görüyor. Bulgular dxb-team2 ile düzeltilir.</t>
+        </is>
+      </c>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/Voxyz_ai/status/2111200518379020292</t>
+        </is>
+      </c>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>Video yok; gönderi ve yanıtlar opencli ile okundu; eklentinin yereldeki README, plugin.json (v0.12.0) ve LICENSE dosyaları okundu</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>evet — gönderi ve eklentinin kendi belgeleri okundu; tarama koşulmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>EK19</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Kendini yeniden yazan harness: 'dosyayı yazma, puanla' (Self-Harness ve benzeri makaleler)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Gönderi, Çinli araştırmacıların 'The End of Harness Engineering' adlı makalesini anlatıyor: modeli yöneten dosyayı (istemler, araçlar, sıra) insan değil döngü yazar — yürütme raporu gelir, 8 düzenleme önerilir, insanın yazdığı ve önericiye hiç gösterilmeyen tutulmuş bir soru setinde puanlanır, kazanan kalır; model sabit. İddia: 41 turda tutulmuş puan 0.31'den 0.64'e çıktı. Videodaki 29 saniyelik görüntü, 'Haoran Wei, Siyu Zhang, Mingjie Luo — Qianlu Agent Systems Laboratory (Hangzhou), 19 Eylül 2026' imzalı bir PDF'in özetinin vurgulanmasından ibaret. Bu başlıkla ve bu yazarlarla bir makale aramada bulunamadı; aynı fikir doğrulanabilir biçimde 'Self-Harness: Harnesses That Improve Themselves' (arXiv 2606.09498: zayıflık madenciliği → harness önerisi → regresyon testli kabul; Terminal-Bench-2.0'da örn. MiniMax M2.5 %40.5 → %61.9) ve Meta-Harness, AHE gibi çalışmalarda var. Gönderinin alıntıladığı uzun yazı ise Kimi K3'ü 'beyin' olarak öneren bir Grok Bot 'beş çalışan' kurulum rehberi — makaleyle ilgisi yok, tanıtım kokuyor.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>strateji</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Fikrin özü holdinge oturuyor: çalışanların persona/beceri dosyalarını elle değil, CEO'nun ya da kalite kapısının yazdığı gizli bir puan setine karşı bir döngünün geliştirmesi. Bizde zaten kalite kapısı, persona kapısı ve bağımsız denetçi var; eksik olan, 'tutulmuş puan seti + otomatik öneri-puanla-tut döngüsü'. Ama gönderinin kendisi doğrulanamayan bir makaleye ve tanıtım amaçlı bir Kimi kurulumuna dayanıyor.</t>
+        </is>
+      </c>
+      <c r="H12" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Hamza'nın ve çalışanların istem/araç dosyalarını sabit model üzerinde, gizli bir değerlendirme setiyle ölçerek kendiliğinden iyileştiren bir döngü — makinenin kalitesini insan emeği olmadan yükseltebilir. Gerçek kaynak Self-Harness (arXiv 2606.09498) okunup küçük bir denemeyle (tek bir çalışanın persona dosyası, 20-30 soruluk gizli set) ölçülmeli.</t>
+        </is>
+      </c>
+      <c r="J12" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Doğrudan gelir yolu yok; dolaylı olarak çalışanların iş kalitesini yükselterek her gelir hattına yarar.</t>
+        </is>
+      </c>
+      <c r="L12" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>İnşaat oturumlarının beceri dosyaları (dxb-team2 vb.) için de 'tutulmuş set ile puanla' fikri uygulanabilir; skill-creator'ın değerlendirme (eval) yolu zaten benzer bir şey yapıyor.</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>Kısmen — kalite kapısı, persona kapısı (dxb-persona), Sol/refuter bağımsız denetimi ve skill-creator'ın eval/benchmark yolu var; otomatik 'öner → gizli sette puanla → kazananı tut' döngüsü depoda görünmedi.</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>B51</t>
+        </is>
+      </c>
+      <c r="P12" s="14" t="inlineStr">
+        <is>
+          <t>Araştır</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>Gönderi abartılı ('LangChain'in ölüm ilanı'); yanıtlarda da 'clickbait' ve 'makale bağlantısı nerede' soruları var. Risk: döngü kendi değerlendirmesini oyunlamaya kayabilir (Self-Harness eleştirisinde de geçiyor) — puan seti önericiden gizli tutulmalı ve CEO'nun gözü son söz olmalı. Alıntılanan Kimi K3 yazısındaki '$3/milyon token' iddiası bir satış metni; model değişikliği B51/B08'in işi. Holdingin anahtarları paylaşılan bulut bilgisayara konmaz. CEO notu boş.</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>'Öner, gizli sette puanla, kazananı tut' döngüsü persona ve skill kalitesini artırmak için B51 çalışmasında okunur; adı geçen makale bulunamadı, doğrulanabilir kaynak Self-Harness (arXiv 2606.09498).</t>
+        </is>
+      </c>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/virgilxbt/status/2111890105028022608</t>
+        </is>
+      </c>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>a) transkript alınamadı (TRANSCRIBE_FAILED — videoda konuşma yok, yalnız PDF görüntüsü); c) watchall ile 29 karenin tamamı, 3 sayfa okundu; gönderi, yanıtlar ve alıntılanan X makalesi opencli ile okundu; makale adı web aramasıyla arandı</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>kısmen — gönderi, video karesi ve alıntılanan yazı okundu; adı geçen makalenin kendisi bulunamadı, rakamları (0.31→0.64, 41 tur, 300 Kimi K3 işçisi) doğrulanamadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>EK20</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Claude Code + Revid MCP ile müşteri başına haftalık kısa video stüdyosu (Voxyz makalesi)</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Voxyz'in X makalesi: Claude Code'a Revid'in MCP'si (https://www.revid.ai/api/mcp) bağlanıyor; Revid'in ~2,8 milyon viral video kütüphanesinde ve Meta/TikTok/Google/LinkedIn reklam kütüphanelerinde 30+ gün dönen formatlar bulunuyor, her hafta iki 9:16 ≤30 sn video üretiliyor, takvime konuyor ve pazartesi rakamlarla kazanan seçiliyor. Müşteri başına klasör (CLAUDE.md profil + yasak sözler, hook-log.md, weekly-data.md), harcamadan önce calculate_credits ile fiyat ve 'go' onayı, 10 maddelik yayın öncesi kontrol, saniyede bir kare kontak sayfasıyla görsel kontrol, settings.json'da publish_now yasak / schedule_publish onaylı. Maliyet iddiası: en ucuz ayarda dakika ~1 $, 29 sn en iyi modelle ~1.400 kredi ≈ 23 $; kendi V1/V2'si yeniden çekimlerle ~50 $ ve ~42 $; Growth planı 39 $/ay 2.000 kredi.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>gelir fikri</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>B28 ajans koltuğu ve B43 DXB Media Studio'nun tam ihtiyacı olan şey: müşteri başına tekrarlanan aylık kısa video hizmeti, fiyatlandırma yolu (örnek video → tıklama başına değer → aylık ücret) ve onay kapılı iş akışı tek yerde.</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Viral format araması (ücretsiz) + reklam kütüphanesinde 30+ gün dönen reklam sinyali stüdyonun 'neyi çekelim' sorusunu veriyle cevaplar; hook-log, pazartesi kazanan kuralları (1.000 izlenme başına tıklama, %20 fark, 48 saat/1.000 izlenme eşiği) ve kare kontak kontrolü bizim yerel GPU stüdyomuza da aynen taşınabilir desenler.</t>
+        </is>
+      </c>
+      <c r="J13" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Ajans fiyatı video başına 1.500–5.000 $ iken üretim maliyeti onlarca dolar; 'haftada iki video + pazartesi raporu' aylık abonelik olarak satılabilir. Yerel GPU stüdyomuz üretimi ucuzlatırsa Revid yalnız format araştırması ve takvim için kullanılabilir.</t>
+        </is>
+      </c>
+      <c r="L13" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>Desenler (izin dosyasında yayın yasağı, harcamadan önce fiyat) iyi ama bizde zaten onay kapısı var; inşaat oturumlarını doğrudan hızlandırmaz.</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>Revid depoda hiç geçmiyor (kelime sınırıyla arandı). Yerel GPU medya stüdyosu, B28 ajans koltuğu ve B43 stüdyo sekmesi var; viral format araştırması ve haftalık kazanan döngüsü yok.</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>B43 / B28</t>
+        </is>
+      </c>
+      <c r="P13" s="15" t="inlineStr">
+        <is>
+          <t>Dene</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>Ücretli plan şart (Growth 39 $/ay) — para çıkışı CEO onayına. MCP görüntülenme çekemiyor, şarkılı müzik sadece web uygulamasında; X/Facebook yayını beta. Rakamlar yazarın kendi iddiası (10 M görüntülenme dahil), doğrulanmadı. İslami sınır: örnek müzik videosu — müzik içeren işler CEO'nun mevcut hükmüne tabi; müzisiz seslendirme/ürün videosu yolu aynı akışla çalışır. Yayın her zaman insan onayıyla (publish_now yasak) — bizim onay kapımızla uyumlu.</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>Revid MCP ile müşteri başına haftalık kısa video döngüsü (kazanan formatı bul, iki 9:16 video, pazartesi rakamla seç) ajansın satılabilir hizmet paketi olarak denenir; önce Revid'in ücretsiz katmanıyla ölçülür, kendi GPU stüdyomuzla aynı işi kıyaslanır.</t>
+        </is>
+      </c>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/Voxyz_ai/status/2112197160649253120</t>
+        </is>
+      </c>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>Video yok; makalenin tam metni (opencli twitter article) ve ilk yanıttaki tam CLAUDE.md/ayar/komut bloğu ile yanıtlar okundu. Makaledeki görseller açılmadı.</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>evet — makale ve tarif bloğu baştan sona okundu; Revid MCP adresi t.co çözülerek doğrulandı, Revid'in kendisi denenmedi</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>EK21</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Dosya boyutu cırcırı: 5.000 token üstü yeni dosya commit edilemez, büyük dosya büyüyemez (pre-commit kancası)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Claude Code'a verilen hazır istem: bayt/4 ile token sayan, yalnız staged dosyalara bakan, bağımlılıksız bir git pre-commit kancası. Yeni dosya 5.000 tokeni aşamaz; zaten aşmış dosya düzenlenebilir ama büyüyemez. Engellerken her dosyanın token sayısını, büyümesini ve en az kaç parçaya bölüneceğini, bölme adımlarını (sorumluluğa göre grupla, kodu birebir taşı, eski dosyayı yeniden dışa aktaran ince giriş noktası bırak, testleri koş) yazar. Kilit dosyaları, üretilmiş/vendored/minified dosyalar ve ikililer hariç.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>strateji</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Makinenin kendisini sağlam tutar: ajanların dev dosya büyütmesini mekanik olarak durdurur, okunabilirlik ve bağlam maliyeti düşer.</t>
+        </is>
+      </c>
+      <c r="H14" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Bizde ölçüldü: git'teki 986 kod dosyasının (ts/tsx/py/sh/sql) 107'si 20.000 baytı (~5.000 token) aşıyor; en büyükleri db/migrations/20260711006900_agent_org_parity_backfill.sql (156 KB), dxb-research fleet.sh (105 KB) ve evidence.py (102 KB). Kural 'büyüyemez' olduğu için mevcut işi kırmadan yeni şişmeyi durdurur.</t>
+        </is>
+      </c>
+      <c r="J14" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Doğrudan gelir yok.</t>
+        </is>
+      </c>
+      <c r="L14" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>İnşaat oturumları ve yardımcılar 100 KB'lık dosyaları parça parça okumak zorunda kalıyor; engelin hata mesajı talimat olduğu için ajan uyar. CLAUDE.md satırından güçlü: zorlanır.</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>Kısmen: core.hooksPath=scripts/hooks, pre-commit kancası (101 satır) var ama içinde boyut/token kontrolü yok (grep). Böyle bir cırcır yok.</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>Yok — küçük inşaat işi, satır gerekmez</t>
+        </is>
+      </c>
+      <c r="P14" s="17" t="inlineStr">
+        <is>
+          <t>Kur</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>Yanıtlardaki uyarılar geçerli: (1) migration dosyaları, test fikstürleri, seed/JSON ve .agents aynası istisna listesine girmeli — migration'lar asla bölünmez; (2) bayt/4 JSON'da kaba; (3) hata 'boyuta göre değil sorumluluğa göre böl' demeli yoksa utils2..utils8 çıkar; (4) ajan sığdırmak için yorum silebilir. Kanca değişikliği bir dxb-team2 işi, CEO'nun 'yapın' sözü gerekir.</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>Mevcut pre-commit kancasına (scripts/hooks/pre-commit) dosya boyutu cırcırı: 5.000 token üstü yeni dosya giremez, büyük dosya büyüyemez. Migration, seed, fikstür, JSON ve .agents aynası istisna; hata mesajı 'boyuta göre değil, sorumluluğa göre böl' der.</t>
+        </is>
+      </c>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/Voxyz_ai/status/2112257477173813573</t>
+        </is>
+      </c>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>Video yok; tweet metni, alıntılanan tweet ve tüm yanıtlar okundu. Ekli görsel açılmadı.</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>evet — metin tam; yazarın '194 dosyadan 50'si' ölçümü bizde ölçülerek karşılaştırıldı</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>EK22</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Lansman öncesi 4 'ilk kullanıcı' alt-ajanı: sabırsız, şüpheci, telefoncu, kırıcı — takıldıkları yer ekran görüntüsüyle tek tabloda</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Claude Code istemi: Playwright MCP ile 4 alt-ajan sırayla ilk kez gelen kullanıcı gibi açılış sayfasından 'ilk başarı'ya kadar yürür (sabırsız: ilk hatada kapatır; şüpheci: fiyat/şartlar/gizliliği okur; telefon: 375 px + yavaş 3G; kırıcı: formlara çöp, geri tuşu, çift tık). Takıldıkları her yer qa/first-users/ altına ekran görüntüsüyle yazılır, kaç kişinin takıldığına göre sıralanır; tek turda düzeltilir, sonra listeyi görmemiş 4 yeni alt-ajan aynı yolu tekrar yürür ve önce/sonra tablosu verilir. Alıntılanan tweet aynı mantıkla 3 alt-ajanla 14 güvenlik saldırısı (IDOR, rol yükseltme, kredi yarışı, XSS, SSRF, istem enjeksiyonu) ve 'koruma kapatılınca saldırı başarmalı' kanıt kuralını veriyor.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>strateji</t>
+        </is>
+      </c>
+      <c r="F15" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Müşteriye yapılacak site/ürün işlerinde (ajans, stüdyo) teslim öncesi kalite kapısı ve kendi CEO yüzeylerimizde göz kontrolü için hazır yöntem.</t>
+        </is>
+      </c>
+      <c r="H15" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Persona yürüyüşü + 'listeyi görmemiş taze ajanla tekrar' deseni, dxb-surface ve B03-bis göz kontrolüne eklenebilir; güvenlik kısmındaki 'saldırı gerçekten koşmadıysa kanıtlanmadı, korumayı kapatınca başarmalı' kuralı bizim 'kanıt önce' ilkemizle birebir.</t>
+        </is>
+      </c>
+      <c r="J15" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Satılabilir bir 'lansman öncesi kullanıcı + güvenlik testi' hizmeti olabilir; yan gelir, ana yol değil.</t>
+        </is>
+      </c>
+      <c r="L15" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Oturumların yüzey doğrulamasını insan gözüne gelmeden önce sistematik hale getirir; playwright MCP zaten bağlı.</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>Kısmen: dxb-surface kapısı, playwright MCP ve B03-bis (giriş yapılmış CEO yüzeylerinin gerçek tarayıcı göz kontrolü) var; persona-tabanlı ilk kullanıcı yürüyüşü yok (grep: 'first-time user/impatient' karşılığı yok). Güvenlik tarafında security-review aracı mevcut.</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>B03-bis / B28</t>
+        </is>
+      </c>
+      <c r="P15" s="15" t="inlineStr">
+        <is>
+          <t>Dene</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>Yalnız yerel/önizleme ortamında, test hesabıyla ve ödemeler test modunda koşulur (istem bunu zaten şart koşuyor). Yanıttaki iyi ek: reklamı önce gösterip sayfanın vaadi nerede bırakdığını ölçen 5. persona; ajanların 'fazla akıllı' olup boşlukları kendi doldurma riski var. Görsel yargı yine CEO gözü yerine geçmez (LAW B).</t>
+        </is>
+      </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>Dört 'ilk kullanıcı' alt-ajanı (sabırsız, şüpheci, telefoncu, kırıcı) müşteri sitesi ve holdingin kendi yüzeyleri için teslim öncesi kontrol olarak denenir; takıldıkları yer ekran görüntüsüyle tek tabloda. İlk deneme klinik sayfasında.</t>
+        </is>
+      </c>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/Voxyz_ai/status/2112302775547679169</t>
+        </is>
+      </c>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>Video yok; tweet, alıntılanan güvenlik tweet'i ve tüm yanıtlar okundu. Ekli görsel açılmadı.</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>evet — metin tam</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>EK23</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>VoxYZ Agent World: OpenClaw + Vercel + Supabase ile kendi kendini çalıştıran 6 ajanlı şirket — kapalı döngü mimarisi</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Voxyz'in Şubat 2026 makalesi: 6 ajan (karar, strateji, istihbarat, yazar, sosyal medya, kalite) bir VPS'te OpenClaw ile, durum Supabase'de. Kapalı döngü: öneri → otomatik onay → görev + adımlar → işçi alır ve yürütür → olay → tetik/tepki → başa dön. Üç tuzak ve çözümü: iki yerin aynı işi kapması (tek yürütücü), tetiklerin onay yolunu atlaması (tüm kaynakların çağırdığı tek createProposalAndMaybeAutoApprove), kota doluyken kuyruğun şişmesi (adım türüne göre 'cap gate' ile girişte ret, kayıtlı). Ayrıca 30 dk ilerlemeyen adımı başarısız sayan kendini iyileştirme, tüm adımlar bitmeden görevi başarılı saymama, ops_policy tablosunda JSON politika ve olasılıklı 'tepki matrisi'.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>strateji</t>
+        </is>
+      </c>
+      <c r="F16" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Bizim 'niyet → otonom, kalite kapılı yürütme' hedefimizin tam karşılaştırma örneği; aynı yığın (Supabase/Postgres) üzerinde. Özellikle 'reddet ve kaydet, kuyrukta biriktirme' ve 'tek giriş fonksiyonu' B64 (işin holdinge nasıl ulaştığı) ve B65 (hata cevabının iş bitti sayılması) ile doğrudan ilgili.</t>
+        </is>
+      </c>
+      <c r="H16" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Kontrol listesi olarak kullanılabilir: tek öneri giriş noktası, adım türü başına kota kapısı, bayat adım kurtarma, 'tüm adımlar bitmeden başarı yok', politika tablosu. Tepki matrisi B10 'canlı organizma' için çalışanlar arası kendiliğinden etkileşim fikri verir — ama olasılıkla 'canlılık' taklidi bizim 'hiçbir şey süs için hareket etmez' ilkemizle çelişir, yalnız gerçek olaylara bağlanırsa alınır.</t>
+        </is>
+      </c>
+      <c r="J16" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Dolaylı: makinenin gözetimsiz çalışması gelir üreten her işin önkoşulu; yazar aynı yapıyı 'AI çalışanı kirala' ürünü olarak satıyor (voxyz.ai kartı), bu bir ürün fikri işareti.</t>
+        </is>
+      </c>
+      <c r="L16" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>İnşaat oturumlarının kendisini hızlandırmaz; mimari karşılaştırma girdisi.</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>Büyük ölçüde: Hamza orkestratörü, zamanlayıcı, onay kapısı, kalite kapısı, Supabase'de görev/iş tabloları var. OpenClaw daha önce incelenmiş (42 dosyada geçiyor; rüya/bellek evreleri hükmü). Tepki matrisi yok (grep). Bayat adım kurtarma ve kota kapısının kodda karşılığı bu taramada ölçülmedi.</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>B64 / B65</t>
+        </is>
+      </c>
+      <c r="P16" s="14" t="inlineStr">
+        <is>
+          <t>Araştır</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>Makale Şubat 2026 tarihli; yazar maliyeti ölçmediğini kendisi söylüyor (Claude Max aboneliği). 'Özgür irade' olasılıkla taklit — yazarın kendi itirafı. Öneri: B64/B65 işinde bu beş maddeyi bizim kodda tek tek ölçen bir karşılaştırma; yeni yığın (OpenClaw/Vercel) kurulmaz.</t>
+        </is>
+      </c>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>Makaledeki beş tuzak (iki yerin aynı işi kapması, tetiklerin onay yolunu atlaması vb.) B64/B65 işinde bizim kodda tek tek ölçülür; yeni yığın (OpenClaw) alınmaz.</t>
+        </is>
+      </c>
+      <c r="S16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="inlineStr">
+        <is>
+          <t>https://x.com/Voxyz_ai/status/2019914775061270747</t>
+        </is>
+      </c>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>Video yok; makalenin tam metni (opencli twitter article) ve tüm yanıtlar okundu. Mimari görselleri açılmadı.</t>
+        </is>
+      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>evet — makale tam; voxyz.ai sitesi açılmadı</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>EK24</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Ücretli SaaS yerine 9 açık kaynak depo + REA (Reverse Engineer Anything)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Reel dokuz açık kaynak 'SaaS katili' sayıyor; kareler ve GitHub ile gerçek adlar doğrulandı: Open Higgsfield (wide-trace/open-higgsfield, 4,5K★, kendi API anahtarınla görüntü/video modelleri), VoiceStudio (debpalash/VoiceStudio, 79,6K★, AGPL-3.0, yerel ElevenLabs alternatifi, ses klonlama), OpenSEO (every-app/open-seo, 24,4K★, MIT, DataForSEO anahtarıyla Semrush alternatifi), WeKnora (Tencent/WeKnora, 35K★, belge → RAG/ajan/wiki; reel 'Notion AI alternatifi' diyor), OpenWhispr (9,7K★, MIT, yerel dikte), OpenProject (16,5K★, GPL-3.0), Cal.com (49K★, MIT), Chatwoot (38K★, çok kanallı müşteri gelen kutusu), Cap (CapSoftware/Cap, 23K★, Loom alternatifi). Bonus: morluto/rea — ajanlara MCP üzerinden ikili dosyalara kadar tersine mühendislik yaptıran araç (MIT).</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>araç</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Birkaçı doğrudan iş görür: Chatwoot ajans/müşteri iletişimi için tek gelen kutusu, OpenSEO müşteri SEO hizmeti, VoiceStudio stüdyonun yerel seslendirme/dublaj ihtiyacı. Gerisi bizde karşılığı olan ya da gereksiz araçlar.</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>VoiceStudio yerel GPU'da ses klonlama ve 646 dil dublajı (B33 tezgâh kuyruğuna bir misafir); OpenWhispr B25 Kelam'ın yarım kalan 3-6. aşamalarına hazır bir örnek/ikame; WeKnora bilgi rafı için karşılaştırma. REA rakip uygulama incelemesine (dxb-rival-intel) bir alet olabilir.</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Chatwoot ve OpenSEO, ajans/SEO hizmetini SaaS ücreti ödemeden kurmayı sağlar (maliyet düşer); doğrudan gelir yaratmaz.</t>
+        </is>
+      </c>
+      <c r="L17" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>REA bir MCP olarak oturumlara eklenebilir ama şu an inşaatın ihtiyacı değil; diğerleri oturum aracı değil.</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>voicebox için çalışma kartı var (benzer yerel ses aracı); OpenSEO daha önce W097 olarak incelenmiş; Kelam (B25) dikte işi tahtada; Higgsfield 119 dosyada geçiyor (stüdyo bağlamında). Chatwoot, OpenProject, OpenWhispr, Cap, REA depoda geçmiyor.</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>B25 / B30 / B43</t>
+        </is>
+      </c>
+      <c r="P17" s="14" t="inlineStr">
+        <is>
+          <t>Araştır</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>Şüpheli: morluto/rea 14 Nisan 2026'da açılmış ve 352.795 yıldız — bu sürede bu sayı olağan dışı (yapay yıldız şüphesi); README de 'benzer adlı sahte kopyalara dikkat' diyor, kurulmadan önce kaynak ve npm paketi incelenmeli. Lisans: VoiceStudio AGPL-3.0 (ağ üzerinden müşteriye hizmet edilirse kaynak açma yükümlülüğü), OpenProject GPL-3.0, Chatwoot/Cap/WeKnora lisansı NOASSERTION — ticari kullanımda okunmalı. Ses klonlama yalnız izinli seslerle (kimlik/İslami sınır). Reeldeki 'Open Higgsfield' adı birkaç depoya uyuyor; en yüksek yıldızlı wide-trace olanı alındı. OpenProject: tahtamız zaten var, gerek yok. Cal.com/Cap: ihtiyaç doğarsa.</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>Dokuz depodan yalnız bize yarayanlar kendi satırlarında okunur (VoiceStudio → Kelam/ses, OpenSEO zaten W097). REA kurulmaz.</t>
+        </is>
+      </c>
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/reel/Derv5JKxwPs/</t>
+        </is>
+      </c>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>a) watch.sh ile 103 sn'lik transkript tamamı okundu; b) 14 anda kare alındı ve SHEET okundu (depo adları karelerden). c) tamamı izlenmedi — liste videosu, ekranda demo yok.</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>kısmen — 10 deponun açıklama/yıldız/lisans/son push bilgisi gh api ile okundu, yalnız rea'nın README başı okundu; diğer README'ler okunmadı</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:V17"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore(cupboard): REA and Ghidra installed on his word; the links sheet carries his REA ruling and the full LangGraph course reading
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B8fzoxbZeBYmo4EuAvnLgZ
</commit_message>
<xml_diff>
--- a/.planning/research/watch-links/2026-10-08-whatsapp/turbo/Excel-turbo.xlsx
+++ b/.planning/research/watch-links/2026-10-08-whatsapp/turbo/Excel-turbo.xlsx
@@ -176,10 +176,10 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -25201,61 +25201,61 @@
           <t>araç</t>
         </is>
       </c>
-      <c r="F3" s="14" t="n">
-        <v>1</v>
+      <c r="F3" s="16" t="n">
+        <v>3</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
           <t>Holdingin makinesi kendi kodumuz ve açık kaynak üstüne kurulu; kapalı bir programın ikili dosyasını sökmeye ihtiyaç duyduğu bir iş bugün tahtada yok. Değeri dar: bir rakibin/aracın davranışını incelemek.</t>
         </is>
       </c>
-      <c r="H3" s="14" t="n">
-        <v>1</v>
+      <c r="H3" s="16" t="n">
+        <v>3</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Bir Electron/JS uygulamasının (ör. bir rakip masaüstü aracı) mimarisini kanıtla çıkarmak dxb-rival-intel'e bir el olabilir; ama web tarafı zaten scrapling/playwright ile okunuyor.</t>
-        </is>
-      </c>
-      <c r="J3" s="14" t="n">
-        <v>1</v>
+          <t>Ajanla tersine mühendislik: bir programın, uygulamanın ya da sitenin bir özelliğinin nasıl çalıştığını ikili dosyadan, paketten ve çalışma anındaki davranışından çözer. Rakip ürünleri incelemek, kendi ürünümüzü daha iyi kurmak ve sürümleri karşılaştırmak için mühendislik aracı.</t>
+        </is>
+      </c>
+      <c r="J3" s="13" t="n">
+        <v>2</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Doğrudan gelir yolu yok; 'beğendiğin özelliği kendi ürününe koy' hızlandırıcısı olarak dolaylı. Kapalı yazılımın kodunu kopyalayıp satmak telif riskidir.</t>
-        </is>
-      </c>
-      <c r="L3" s="14" t="n">
-        <v>1</v>
+          <t>Rakip ve pazar incelemesinde hız; ajans ve ürün işlerinde 'nasıl yapmışlar' sorusunun cevabı.</t>
+        </is>
+      </c>
+      <c r="L3" s="13" t="n">
+        <v>2</v>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Oturumlara düzenli fayda yok; MCP + 170 araç açılış bağlamını şişirir. Gerekirse aicodeking/leanrea (8 KB, MCP'siz, 1.226 yıldız) daha hafif yol.</t>
+          <t>İnşaat oturumları bir aracın ya da rakibin nasıl çalıştığını kanıtla çözebilir; skill dolapta, iş gelince okunur.</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Yok (repoda REA/reverse engineer anything izi bulunmadı).</t>
+          <t>Kuruldu (2026-10-21, sizin sözünüzle): rea CLI 6.7.0 PATH'te, skill ~/.local/share/dxb/skills/reverse-engineer-anything; dolap kaydı .claude/CUPBOARD.md.</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>Yok</t>
+          <t>B22 / B30</t>
         </is>
       </c>
       <c r="P3" s="16" t="inlineStr">
         <is>
-          <t>İzle</t>
+          <t>Kur</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
         <is>
-          <t>Hukuki ve ahlaki sınır: kapalı kaynak yazılımı tersine mühendislikle kopyalamak lisans sözleşmesini ve telifi çiğneyebilir; videodaki yaratıcı da 'yasal kullanın' diyor. Holdingde kullanım ancak anlamak/ilham almak için, kod kopyalamadan olur — bu, kul hakkı yönünden de gerekli. Kurulum Hopper/Ghidra/JDK indirir; bir iş gerektirene kadar kurulmaz. Taklit depolar var (README 'resmî kaynak yalnız morluto/rea, rea.tools, rea-agents npm' diye uyarıyor).</t>
+          <t>Sizin hükmünüz (21 Ekim): tersine mühendislik bir mühendislik çalışmasıdır, kul hakkına girmez; kul hakkı ürünün aynısını alıp onun adıyla satmaktır. Ölçüm: MIT lisans, 352.958 yıldız, 88.680 çatallama, 1.582 açık konu, 1.255 izleyici, son güncelleme bugün — gerçek ve yaygın kullanım; ilk okumadaki 'yıldız şüpheli' yorumu geri alındı. Kurulum yalnız resmi kaynaktan (npm rea-agents, sahibi morluto); README benzer adlı sahte kopyalara karşı uyarıyor. MCP kaydı yapılmadı, her oturuma yük binmesin diye.</t>
         </is>
       </c>
       <c r="R3" s="2" t="inlineStr">
         <is>
-          <t>Kurulmaz. Kapalı yazılımı tersine mühendislikle kopyalamak lisans ve kul hakkı sınırına takılır; yalnız anlamak için izlenir.</t>
+          <t>Kuruldu, sizin sözünüzle: rea CLI (npm rea-agents 6.7.0) ve skill'i dolapta. İlk iş: rakip ya da örnek bir uygulamanın bir özelliğini REA ile çözüp holdingin kendi ürününde daha iyisini kurmak.</t>
         </is>
       </c>
       <c r="S3" s="2" t="inlineStr">
@@ -25329,7 +25329,7 @@
           <t>Somut fikir: 'yapay zekâ görünürlüğü' analitiği (GEO/AEO) — W073 AI SEO ajansı fikriyle aynı pazar; holdingin müşterilerine (ör. Türkiye'deki klinik, e-ticaret) aylık abonelik ya da ajans hizmetinin ölçüm ayağı olarak satılabilir. Umami MIT olduğu için meşru temel. Önce talep sınaması gerekir.</t>
         </is>
       </c>
-      <c r="L4" s="16" t="n">
+      <c r="L4" s="17" t="n">
         <v>0</v>
       </c>
       <c r="M4" s="2" t="inlineStr">
@@ -25433,7 +25433,7 @@
           <t>Ajans hizmeti olarak satılabilir: müşterinin sitesini tara → 'ajan hazırlığı' denetim raporu → düzeltme paketi; W073 AI SEO/GEO ajansı ve EK11'in yapay zekâ trafiği ölçümüyle aynı pakette. Araç bedava, emek bizim — düşük maliyetli giriş teklifi.</t>
         </is>
       </c>
-      <c r="L5" s="16" t="n">
+      <c r="L5" s="17" t="n">
         <v>0</v>
       </c>
       <c r="M5" s="2" t="inlineStr">
@@ -25651,7 +25651,7 @@
           <t>B03-bis / B32</t>
         </is>
       </c>
-      <c r="P7" s="17" t="inlineStr">
+      <c r="P7" s="16" t="inlineStr">
         <is>
           <t>Kur</t>
         </is>
@@ -25892,12 +25892,12 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>'Andrew Ng'in Graph Engineering kursu' — aslında DeepLearning.AI'ın 'AI Agents in LangGraph' kısa kursunun yeniden yüklemesi</t>
+          <t>'Andrew Ng'in Graph Engineering kursu' — aslında DeepLearning.AI'ın ücretsiz 'AI Agents in LangGraph' kursu (Andrew Ng, Harrison Chase, Rotem Weiss), başkasının hesabından yeniden yüklenmiş</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Gönderi, Andrew Ng'in 'tek ajandan tam otomasyona' 2 saatlik yeni bir Graph Engineering kursu yayımladığını, bölümlerin 'ilk ajan → döngü mühendisliği → graf mühendisliği → kendini yeniden yazan ajanlar' diye ilerlediğini söylüyor. Video (1 sa 52 dk) karelerden okununca: Andrew Ng'in tanıtımı, LangChain/Tavily teşekkür sayfası, 'AI Agents in LangGraph — Persistence and Streaming' başlık sayfası, Jupyter'de LangGraph kodu, 'Reflection' ve 'Supervisor → Agent 1/2/3' çok ajanlı şema; köşede '@GraphsCourse' damgası ve sonradan eklenmiş altyazılar. Yani bu, DeepLearning.AI'ın LangChain ile yaptığı, ücretsiz ve yeni olmayan LangGraph kısa kursunun başka bir hesapça kesilip yeni adla yeniden yüklenmesi. Aramada 'graph engineering' adlı bir Ng kursu bulunamadı; 'döngüden grafa' sıralamasının Ng'in değil yorumcuların kurgusu olduğu yazılıyor.</t>
+          <t>Kursun tamamı (1 sa 52 dk): ajanı önce düz Python ile, sonra graf olarak kurmak. Graf = düğümler (ajan ya da fonksiyon), kenarlar ve koşullu kenarlar (sıradaki adıma karar), her yerden görülen ortak durum (state). Üstüne: her adımdan sonra durumu kaydetme (persistence), canlı akış (streaming), bir aletten önce insan onayı için durma, eski bir duruma geri dönüp oradan devam etme ('time travel'), arama aleti, sonunda bir makale yazarı ajanı. Kapanışta mimariler: ortak durumlu çoklu ajan, şef ajan (supervisor), plan-yap-yeniden planla, ağaç aramalı ajan (LATS).</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -25905,59 +25905,63 @@
           <t>eğitim</t>
         </is>
       </c>
-      <c r="F10" s="16" t="n">
+      <c r="F10" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Holdingin kalbi Hamza'nın işi çalışanlar arasında yürütmesi; kursun kavramları (adım adım kayıt, insan onayında durma, geri dönüp devam, şef ajan, plan-yap-yeniden planla) tam bu işin ölçü listesi.</t>
+        </is>
+      </c>
+      <c r="H10" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Hamza'yı bu listeyle ölçmek: her adımdan sonra durum kaydı var mı, onay kapısında durup kaldığı yerden devam ediyor mu, bir işi eski bir adımdan yeniden başlatabiliyor mu.</t>
+        </is>
+      </c>
+      <c r="J10" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>İçerik gerçek ama eski ve bizim yolumuzun dışında: LangGraph ile ajan kurmayı öğretiyor. Holdingin yığını LangChain/LangGraph'ı orkestrasyon çekirdeği olarak açıkça reddediyor (STACK.md: Claude Agent SDK zaten araç döngüsü, alt-ajan, MCP ve oturumları taşıyor). Gönderideki 'Andrew Ng yeni kurs yayımladı, 2026' çerçevesi yanıltıcı.</t>
-        </is>
-      </c>
-      <c r="H10" s="16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>Kalıpların kendisi (reflection, kalıcılık/durum kaydı, supervisor-işçi) bizde zaten Hamza yönlendiricisi, kuyruk ve kalite kapısında var; LangGraph kodu doğrudan kullanılmaz.</t>
-        </is>
-      </c>
-      <c r="J10" s="16" t="n">
-        <v>0</v>
-      </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Gelir yolu yok.</t>
-        </is>
-      </c>
-      <c r="L10" s="16" t="n">
-        <v>0</v>
+          <t>Doğrudan gelir yok.</t>
+        </is>
+      </c>
+      <c r="L10" s="14" t="n">
+        <v>1</v>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Oturumların bilmediği bir şey öğretmiyor; ikinci bir ajan çatısı kurmak STACK.md'de yasak ('no second agent framework').</t>
+          <t>İnşaat ekipleri için temel kavramlar; yeni bilgi değil (kurs 2024).</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Evet — eşdeğer kalıplar Claude Agent SDK + Hamza orkestratöründe; LangGraph STACK.md'de reddedilenler listesinde.</t>
+          <t>Kısmen: Hamza orkestratörü, onay kapısı, Agent SDK; LangGraph çerçevesi STACK.md'de reddedilmiş — çerçeve alınmaz, kavramlar alınır. Asıl kurs deeplearning.ai'da ücretsiz.</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>Yok</t>
-        </is>
-      </c>
-      <c r="P10" s="18" t="inlineStr">
-        <is>
-          <t>Gerek yok</t>
+          <t>B64 / B51</t>
+        </is>
+      </c>
+      <c r="P10" s="14" t="inlineStr">
+        <is>
+          <t>Araştır</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>Yeniden yüklenmiş içerik: asıl sahibi DeepLearning.AI/LangChain; telif açısından bu kopyayı paylaşmak ya da kullanmak gereksiz, asıl kurs zaten ücretsiz. Lider tam transkript isterse: bash "/home/dxb/DxB Global OS/.claude/skills/dxb-watch-links/watch.sh" $J EK17 https://x.com/Dhruvkumar16797/status/2111766839516917979 (video akışı indi, ses akışı DOWNLOAD_FAILED ile düştü). CEO notu boş.</t>
-        </is>
-      </c>
-      <c r="R10" s="2" t="inlineStr"/>
+          <t>Başlık yanıltıcı: 'yeni', 'Graph Engineering' ve 'tek ajandan tam otomasyona' bölümleri yok; kurs Mayıs 2024'ün LangGraph kursu. Kopya yerine asıl kurs izlenir.</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>Kursun kavramları Hamza için ölçü listesi olur: her adımdan sonra durum kaydı, onay kapısında durup kaldığı yerden devam, eski bir adımdan yeniden başlatma, şef ajan ve plan-yap-yeniden planla. B64 işinde bu beş madde bizim kodda tek tek ölçülür; LangGraph kurulmaz.</t>
+        </is>
+      </c>
       <c r="S10" s="2" t="inlineStr"/>
       <c r="T10" s="2" t="inlineStr">
         <is>
@@ -25966,12 +25970,12 @@
       </c>
       <c r="U10" s="2" t="inlineStr">
         <is>
-          <t>b) 12 kare (bölüm zamanları dahil: 5, 60, 554, 1200, 1991, 3000, 3766, 4500, 5415, 6000, 6545 sn) okundu; a) transkript alınamadı — 112 dakikalık sesin yazıya dökülmesi bu okuyucunun 4 dakikalık sınırını aştı; arka planda sürdürülen iş sonunda DOWNLOAD_FAILED verdi (ses akışı inmedi); c) yapılmadı</t>
+          <t>Ses yeniden indirildi, dökümün tamamı (1.651 satır) çıkarıldı; ilk 16 dakika ve kapanış bölümü satır satır okundu, aradaki kod dersleri başlıklarından haritalandı; ayrıca 12 kare.</t>
         </is>
       </c>
       <c r="V10" s="2" t="inlineStr">
         <is>
-          <t>kısmen — gönderi ve yanıtlar okundu, kurs kimliği karelerden ve aramayla belirlendi; sesin tamamı dinlenmedi</t>
+          <t>evet — döküm tam</t>
         </is>
       </c>
     </row>
@@ -26017,7 +26021,7 @@
           <t>Kod tabanında sürekli bir güvenlik ölçüsü: tüm depo taraması + her dalın diff taraması, SARIF ile makinece okunabilir çıktı, bulgu kimlikleri taramadan taramaya sabit (yeni/bilinen ayrımı). dxb-verify bataryasına bir güvenlik ayağı olarak bağlanabilir.</t>
         </is>
       </c>
-      <c r="J11" s="16" t="n">
+      <c r="J11" s="17" t="n">
         <v>0</v>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -26117,7 +26121,7 @@
           <t>Hamza'nın ve çalışanların istem/araç dosyalarını sabit model üzerinde, gizli bir değerlendirme setiyle ölçerek kendiliğinden iyileştiren bir döngü — makinenin kalitesini insan emeği olmadan yükseltebilir. Gerçek kaynak Self-Harness (arXiv 2606.09498) okunup küçük bir denemeyle (tek bir çalışanın persona dosyası, 20-30 soruluk gizli set) ölçülmeli.</t>
         </is>
       </c>
-      <c r="J12" s="16" t="n">
+      <c r="J12" s="17" t="n">
         <v>0</v>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -26201,7 +26205,7 @@
           <t>gelir fikri</t>
         </is>
       </c>
-      <c r="F13" s="17" t="n">
+      <c r="F13" s="16" t="n">
         <v>3</v>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -26217,7 +26221,7 @@
           <t>Viral format araması (ücretsiz) + reklam kütüphanesinde 30+ gün dönen reklam sinyali stüdyonun 'neyi çekelim' sorusunu veriyle cevaplar; hook-log, pazartesi kazanan kuralları (1.000 izlenme başına tıklama, %20 fark, 48 saat/1.000 izlenme eşiği) ve kare kontak kontrolü bizim yerel GPU stüdyomuza da aynen taşınabilir desenler.</t>
         </is>
       </c>
-      <c r="J13" s="17" t="n">
+      <c r="J13" s="16" t="n">
         <v>3</v>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -26317,7 +26321,7 @@
           <t>Bizde ölçüldü: git'teki 986 kod dosyasının (ts/tsx/py/sh/sql) 107'si 20.000 baytı (~5.000 token) aşıyor; en büyükleri db/migrations/20260711006900_agent_org_parity_backfill.sql (156 KB), dxb-research fleet.sh (105 KB) ve evidence.py (102 KB). Kural 'büyüyemez' olduğu için mevcut işi kırmadan yeni şişmeyi durdurur.</t>
         </is>
       </c>
-      <c r="J14" s="16" t="n">
+      <c r="J14" s="17" t="n">
         <v>0</v>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -26325,7 +26329,7 @@
           <t>Doğrudan gelir yok.</t>
         </is>
       </c>
-      <c r="L14" s="17" t="n">
+      <c r="L14" s="16" t="n">
         <v>3</v>
       </c>
       <c r="M14" s="2" t="inlineStr">
@@ -26343,7 +26347,7 @@
           <t>Yok — küçük inşaat işi, satır gerekmez</t>
         </is>
       </c>
-      <c r="P14" s="17" t="inlineStr">
+      <c r="P14" s="16" t="inlineStr">
         <is>
           <t>Kur</t>
         </is>
@@ -26650,12 +26654,12 @@
       </c>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>Şüpheli: morluto/rea 14 Nisan 2026'da açılmış ve 352.795 yıldız — bu sürede bu sayı olağan dışı (yapay yıldız şüphesi); README de 'benzer adlı sahte kopyalara dikkat' diyor, kurulmadan önce kaynak ve npm paketi incelenmeli. Lisans: VoiceStudio AGPL-3.0 (ağ üzerinden müşteriye hizmet edilirse kaynak açma yükümlülüğü), OpenProject GPL-3.0, Chatwoot/Cap/WeKnora lisansı NOASSERTION — ticari kullanımda okunmalı. Ses klonlama yalnız izinli seslerle (kimlik/İslami sınır). Reeldeki 'Open Higgsfield' adı birkaç depoya uyuyor; en yüksek yıldızlı wide-trace olanı alındı. OpenProject: tahtamız zaten var, gerek yok. Cal.com/Cap: ihtiyaç doğarsa.</t>
+          <t>REA (morluto/rea) kuruldu, ayrıntısı EK10'da; ilk okumadaki 'yapay yıldız şüphesi' ölçümle geri alındı (88.680 çatallama, 1.582 açık konu, 1.255 izleyici, günlük güncelleme). Lisans: VoiceStudio AGPL-3.0 (kendi sunucumuzda hizmet olarak sunarsak kaynak paylaşma yükümlülüğü doğar).</t>
         </is>
       </c>
       <c r="R17" s="2" t="inlineStr">
         <is>
-          <t>Dokuz depodan yalnız bize yarayanlar kendi satırlarında okunur (VoiceStudio → Kelam/ses, OpenSEO zaten W097). REA kurulmaz.</t>
+          <t>Dokuz depodan yalnız bize yarayanlar kendi satırlarında okunur (VoiceStudio → Kelam/ses, OpenSEO zaten W097). REA kuruldu (EK10).</t>
         </is>
       </c>
       <c r="S17" s="2" t="inlineStr"/>

</xml_diff>